<commit_message>
experimental new damper logic
</commit_message>
<xml_diff>
--- a/docs/damping_curve.xlsx
+++ b/docs/damping_curve.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\un1corn\UserSpace\Games\Steam_Library\steamapps\common\BeamNG_Userdata\current\mods\unpacked\un1corn_qlourie_astral_r\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\mods\unpacked\un1corn_qlourie_astral_r\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61AA2477-6E76-484F-B0B2-0B0FA72C70D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LSC Sweep" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
total revamp of damping calculation logic
</commit_message>
<xml_diff>
--- a/docs/damping_curve.xlsx
+++ b/docs/damping_curve.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\mods\unpacked\un1corn_qlourie_astral_r\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61AA2477-6E76-484F-B0B2-0B0FA72C70D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A16FF841-20CB-4218-B4EA-75B068F89C8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LSC Sweep" sheetId="1" r:id="rId1"/>
@@ -18,8 +18,9 @@
     <sheet name="LSR Sweep" sheetId="5" r:id="rId3"/>
     <sheet name="Full Sweep" sheetId="3" r:id="rId4"/>
     <sheet name="Parameters" sheetId="4" r:id="rId5"/>
+    <sheet name="Calculator" sheetId="6" r:id="rId6"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" forceFullCalc="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="145">
   <si>
     <t>Astral · LSC sweep</t>
   </si>
@@ -306,9 +307,6 @@
     <t>HSC 越接近 0，第二膝点越晚、附加斜率越大；曲线交叉按公式保留。</t>
   </si>
   <si>
-    <t>来源：研究会话 v13；当前修订：k2 为 0.52～0.68，取消 HSC 中间段倍率（2026-09-20）。</t>
-  </si>
-  <si>
     <t>chatgpt-conversation://6a9ed043-7848-83e8-9d36-6e63c8202898</t>
   </si>
   <si>
@@ -350,16 +348,143 @@
   <si>
     <t>采样：0～1.00 m/s，每 0.05 m/s 一点，共 21 点；不另加膝点采样。</t>
   </si>
+  <si>
+    <t>当前 Type-A：k1 0.12/0.15/0.17；rL 0.78～0.90；k2 0.58～0.62（2026-09-28）。</t>
+  </si>
+  <si>
+    <t>Astral · Type-A 阻尼计算器</t>
+  </si>
+  <si>
+    <t>输入</t>
+  </si>
+  <si>
+    <t>数值</t>
+  </si>
+  <si>
+    <t>范围 / 单位</t>
+  </si>
+  <si>
+    <t>阻尼力大小</t>
+  </si>
+  <si>
+    <t>结果</t>
+  </si>
+  <si>
+    <t>车型</t>
+  </si>
+  <si>
+    <t>Rally2</t>
+  </si>
+  <si>
+    <t>砂石 Type-A</t>
+  </si>
+  <si>
+    <t>压缩</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>LSC / c</t>
+  </si>
+  <si>
+    <t>回弹</t>
+  </si>
+  <si>
+    <t>HSC / C</t>
+  </si>
+  <si>
+    <t>−20～0 格</t>
+  </si>
+  <si>
+    <t>LSR / R</t>
+  </si>
+  <si>
+    <t>当前曲线系数</t>
+  </si>
+  <si>
+    <t>轴速大小</t>
+  </si>
+  <si>
+    <t>LS 压缩 cL</t>
+  </si>
+  <si>
+    <t>中间段 cM</t>
+  </si>
+  <si>
+    <t>HS 附加段 A</t>
+  </si>
+  <si>
+    <t>合计 HS 压缩 cH</t>
+  </si>
+  <si>
+    <t>格数与映射</t>
+  </si>
+  <si>
+    <t>说明</t>
+  </si>
+  <si>
+    <t>LS 回弹</t>
+  </si>
+  <si>
+    <t>HS 回弹</t>
+  </si>
+  <si>
+    <t>c 总格数</t>
+  </si>
+  <si>
+    <t>−格数～0</t>
+  </si>
+  <si>
+    <t>R 总格数</t>
+  </si>
+  <si>
+    <t>c 标准位置</t>
+  </si>
+  <si>
+    <t>映射至 −20～0</t>
+  </si>
+  <si>
+    <t>C 标准位置</t>
+  </si>
+  <si>
+    <t>−20～0</t>
+  </si>
+  <si>
+    <t>R 标准位置</t>
+  </si>
+  <si>
+    <t>映射至 −40～0</t>
+  </si>
+  <si>
+    <t>c 插值区间</t>
+  </si>
+  <si>
+    <t>C 插值区间</t>
+  </si>
+  <si>
+    <t>R 插值区间</t>
+  </si>
+  <si>
+    <t>黄色格可输入；换车型后，请将 c／R 调整到该车型的有效范围。</t>
+  </si>
+  <si>
+    <t>0 为最硬端；两项输出均为同一轴速下的力大小，不使用回弹图的负号。</t>
+  </si>
+  <si>
+    <t>按连续分段接续模型计算，未计入 LRS／DSV、限位、弹簧与气体力。</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
+    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="176" formatCode="0.000"/>
     <numFmt numFmtId="177" formatCode="0.0"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="13">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -407,8 +532,46 @@
       <family val="3"/>
       <charset val="134"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF24364B"/>
+      <name val="Microsoft YaHei"/>
+      <family val="2"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color rgb="FF24364B"/>
+      <name val="Microsoft YaHei"/>
+      <family val="2"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color rgb="FF24364B"/>
+      <name val="Microsoft YaHei"/>
+      <family val="2"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Microsoft YaHei"/>
+      <family val="2"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF566578"/>
+      <name val="Microsoft YaHei"/>
+      <family val="2"/>
+      <charset val="134"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -450,8 +613,21 @@
         <fgColor rgb="FFE8EDF3"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF30475E"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -468,12 +644,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
+    <xf numFmtId="41" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
@@ -545,10 +731,21 @@
     <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="2" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="2" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="2" xfId="2" applyFont="1" applyFill="1"/>
+    <xf numFmtId="1" fontId="8" fillId="10" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="8" fillId="10" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="8" fillId="9" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="10" fillId="9" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="176" fontId="8" fillId="9" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="2" xfId="2" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="2" xfId="2" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Normal" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
     <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="千位分隔[0]" xfId="2" builtinId="6"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -697,61 +894,61 @@
                   <c:v>65</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>126.36000000000001</c:v>
+                  <c:v>130</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>173.16</c:v>
+                  <c:v>186.42</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>219.96</c:v>
+                  <c:v>237.12</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>266.76</c:v>
+                  <c:v>287.82</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>313.56</c:v>
+                  <c:v>338.52</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>360.36</c:v>
+                  <c:v>389.21999999999997</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>407.16</c:v>
+                  <c:v>439.92</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>453.96</c:v>
+                  <c:v>490.62</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>500.76000000000005</c:v>
+                  <c:v>541.31999999999994</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>547.56000000000006</c:v>
+                  <c:v>592.02</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>594.36</c:v>
+                  <c:v>642.72</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>766.1600000000002</c:v>
+                  <c:v>818.42000000000019</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>937.96</c:v>
+                  <c:v>994.11999999999989</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>1109.76</c:v>
+                  <c:v>1169.8200000000002</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>1281.5600000000002</c:v>
+                  <c:v>1345.5200000000002</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>1453.3600000000001</c:v>
+                  <c:v>1521.22</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>1625.1600000000003</c:v>
+                  <c:v>1696.92</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>1796.96</c:v>
+                  <c:v>1872.62</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>1968.76</c:v>
+                  <c:v>2048.3200000000002</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -868,58 +1065,58 @@
                   <c:v>190</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>264.48</c:v>
+                  <c:v>279.58499999999998</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>336.68000000000006</c:v>
+                  <c:v>356.53499999999997</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>408.88</c:v>
+                  <c:v>433.48500000000001</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>481.08</c:v>
+                  <c:v>510.43499999999995</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>553.28</c:v>
+                  <c:v>587.38499999999999</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>625.48</c:v>
+                  <c:v>664.33500000000004</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>697.68000000000006</c:v>
+                  <c:v>741.28500000000008</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>769.88</c:v>
+                  <c:v>818.23500000000001</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>842.08</c:v>
+                  <c:v>895.18500000000006</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>914.28</c:v>
+                  <c:v>972.13499999999999</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>1111.48</c:v>
+                  <c:v>1174.085</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>1308.6799999999998</c:v>
+                  <c:v>1376.0349999999999</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>1505.88</c:v>
+                  <c:v>1577.9850000000001</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>1703.0800000000002</c:v>
+                  <c:v>1779.9350000000002</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>1900.28</c:v>
+                  <c:v>1981.885</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>2097.48</c:v>
+                  <c:v>2183.835</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>2294.6800000000003</c:v>
+                  <c:v>2385.7849999999999</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>2491.88</c:v>
+                  <c:v>2587.7349999999997</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1036,58 +1233,58 @@
                   <c:v>250</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>360</c:v>
+                  <c:v>375</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>460</c:v>
+                  <c:v>480</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>560</c:v>
+                  <c:v>585</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>660</c:v>
+                  <c:v>690</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>760</c:v>
+                  <c:v>795</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>860</c:v>
+                  <c:v>900</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>960</c:v>
+                  <c:v>1005.0000000000001</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1060</c:v>
+                  <c:v>1110</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>1160</c:v>
+                  <c:v>1215</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>1260</c:v>
+                  <c:v>1320</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>1485</c:v>
+                  <c:v>1550</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>1710</c:v>
+                  <c:v>1779.9999999999998</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>1935</c:v>
+                  <c:v>2010</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>2160</c:v>
+                  <c:v>2240</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>2385</c:v>
+                  <c:v>2470</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>2610</c:v>
+                  <c:v>2700</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>2835</c:v>
+                  <c:v>2930</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>3060</c:v>
+                  <c:v>3160</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1204,58 +1401,58 @@
                   <c:v>310</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>462.52</c:v>
+                  <c:v>465</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>592.72</c:v>
+                  <c:v>603.88</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>722.92000000000007</c:v>
+                  <c:v>738.73</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>853.12000000000012</c:v>
+                  <c:v>873.57999999999993</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>983.31999999999994</c:v>
+                  <c:v>1008.43</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1113.5200000000002</c:v>
+                  <c:v>1143.2800000000002</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>1243.7200000000003</c:v>
+                  <c:v>1278.1300000000001</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1373.92</c:v>
+                  <c:v>1412.98</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>1504.1200000000003</c:v>
+                  <c:v>1547.83</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>1634.3200000000002</c:v>
+                  <c:v>1682.6799999999998</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>1889.5200000000004</c:v>
+                  <c:v>1942.5300000000002</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>2144.7199999999998</c:v>
+                  <c:v>2202.3799999999997</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>2399.9200000000005</c:v>
+                  <c:v>2462.23</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>2655.1200000000003</c:v>
+                  <c:v>2722.08</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>2910.32</c:v>
+                  <c:v>2981.93</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>3165.5200000000004</c:v>
+                  <c:v>3241.7799999999997</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>3420.7200000000003</c:v>
+                  <c:v>3501.6299999999997</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>3675.9200000000005</c:v>
+                  <c:v>3761.48</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1375,55 +1572,55 @@
                   <c:v>555</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>726.68</c:v>
+                  <c:v>728.9</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>889.48</c:v>
+                  <c:v>895.4</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1052.28</c:v>
+                  <c:v>1061.8999999999999</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1215.08</c:v>
+                  <c:v>1228.3999999999999</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1377.88</c:v>
+                  <c:v>1394.9</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>1540.68</c:v>
+                  <c:v>1561.4</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1703.4799999999998</c:v>
+                  <c:v>1727.8999999999999</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>1866.28</c:v>
+                  <c:v>1894.4</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>2029.0799999999997</c:v>
+                  <c:v>2060.8999999999996</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>2316.88</c:v>
+                  <c:v>2352.3999999999996</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>2604.6799999999998</c:v>
+                  <c:v>2643.8999999999996</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>2892.4799999999996</c:v>
+                  <c:v>2935.3999999999996</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>3180.28</c:v>
+                  <c:v>3226.9</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>3468.08</c:v>
+                  <c:v>3518.3999999999996</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>3755.88</c:v>
+                  <c:v>3809.9</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>4043.68</c:v>
+                  <c:v>4101.3999999999996</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>4331.4799999999996</c:v>
+                  <c:v>4392.8999999999996</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1741,58 +1938,58 @@
                   <c:v>250</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>360</c:v>
+                  <c:v>375</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>460</c:v>
+                  <c:v>480</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>560</c:v>
+                  <c:v>585</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>660</c:v>
+                  <c:v>690</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>760</c:v>
+                  <c:v>795</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>860</c:v>
+                  <c:v>900</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>960</c:v>
+                  <c:v>1005.0000000000001</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1060</c:v>
+                  <c:v>1110</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>1160</c:v>
+                  <c:v>1215</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>1300</c:v>
+                  <c:v>1340</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>1450</c:v>
+                  <c:v>1495</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>1600</c:v>
+                  <c:v>1649.9999999999998</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>1750</c:v>
+                  <c:v>1805</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>1900</c:v>
+                  <c:v>1960</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>2050</c:v>
+                  <c:v>2115</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>2200</c:v>
+                  <c:v>2270</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>2350</c:v>
+                  <c:v>2425</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>2500</c:v>
+                  <c:v>2580</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1909,58 +2106,58 @@
                   <c:v>250</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>360</c:v>
+                  <c:v>375</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>460</c:v>
+                  <c:v>480</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>560</c:v>
+                  <c:v>585</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>660</c:v>
+                  <c:v>690</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>760</c:v>
+                  <c:v>795</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>860</c:v>
+                  <c:v>900</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>960</c:v>
+                  <c:v>1005.0000000000001</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1060</c:v>
+                  <c:v>1110</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>1160</c:v>
+                  <c:v>1215</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>1295</c:v>
+                  <c:v>1337.5</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>1482.5</c:v>
+                  <c:v>1530</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>1670</c:v>
+                  <c:v>1722.4999999999998</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>1857.5</c:v>
+                  <c:v>1915</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>2045.0000000000002</c:v>
+                  <c:v>2107.5</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>2232.5</c:v>
+                  <c:v>2300</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>2420</c:v>
+                  <c:v>2492.5</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>2607.5</c:v>
+                  <c:v>2685</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>2795</c:v>
+                  <c:v>2877.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2077,58 +2274,58 @@
                   <c:v>250</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>360</c:v>
+                  <c:v>375</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>460</c:v>
+                  <c:v>480</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>560</c:v>
+                  <c:v>585</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>660</c:v>
+                  <c:v>690</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>760</c:v>
+                  <c:v>795</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>860</c:v>
+                  <c:v>900</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>960</c:v>
+                  <c:v>1005.0000000000001</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1060</c:v>
+                  <c:v>1110</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>1160</c:v>
+                  <c:v>1215</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>1260</c:v>
+                  <c:v>1320</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>1485</c:v>
+                  <c:v>1550</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>1710</c:v>
+                  <c:v>1779.9999999999998</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>1935</c:v>
+                  <c:v>2010</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>2160</c:v>
+                  <c:v>2240</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>2385</c:v>
+                  <c:v>2470</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>2610</c:v>
+                  <c:v>2700</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>2835</c:v>
+                  <c:v>2930</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>3060</c:v>
+                  <c:v>3160</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2245,58 +2442,58 @@
                   <c:v>250</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>360</c:v>
+                  <c:v>375</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>460</c:v>
+                  <c:v>480</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>560</c:v>
+                  <c:v>585</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>660</c:v>
+                  <c:v>690</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>760</c:v>
+                  <c:v>795</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>860</c:v>
+                  <c:v>900</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>960</c:v>
+                  <c:v>1005.0000000000001</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1060</c:v>
+                  <c:v>1110</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>1160</c:v>
+                  <c:v>1215</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>1260</c:v>
+                  <c:v>1320</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>1457.5</c:v>
+                  <c:v>1555</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>1720</c:v>
+                  <c:v>1822.4999999999995</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>1982.5</c:v>
+                  <c:v>2090</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>2245</c:v>
+                  <c:v>2357.5</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>2507.5</c:v>
+                  <c:v>2625</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>2770</c:v>
+                  <c:v>2892.5</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>3032.5</c:v>
+                  <c:v>3160</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>3295</c:v>
+                  <c:v>3427.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2413,58 +2610,58 @@
                   <c:v>250</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>360</c:v>
+                  <c:v>375</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>460</c:v>
+                  <c:v>480</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>560</c:v>
+                  <c:v>585</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>660</c:v>
+                  <c:v>690</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>760</c:v>
+                  <c:v>795</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>860</c:v>
+                  <c:v>900</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>960</c:v>
+                  <c:v>1005.0000000000001</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1060</c:v>
+                  <c:v>1110</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>1160</c:v>
+                  <c:v>1215</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>1260</c:v>
+                  <c:v>1320</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>1400</c:v>
+                  <c:v>1545</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>1699.9999999999998</c:v>
+                  <c:v>1849.9999999999995</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>2000</c:v>
+                  <c:v>2155</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>2300</c:v>
+                  <c:v>2460</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>2600</c:v>
+                  <c:v>2765</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>2900</c:v>
+                  <c:v>3070</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>3200</c:v>
+                  <c:v>3375</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>3500</c:v>
+                  <c:v>3680</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3813,61 +4010,61 @@
                   <c:v>65</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>126.36000000000001</c:v>
+                  <c:v>130</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>173.16</c:v>
+                  <c:v>186.42</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>219.96</c:v>
+                  <c:v>237.12</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>266.76</c:v>
+                  <c:v>287.82</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>313.56</c:v>
+                  <c:v>338.52</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>360.36</c:v>
+                  <c:v>389.21999999999997</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>407.16</c:v>
+                  <c:v>439.92</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>453.96</c:v>
+                  <c:v>490.62</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>500.76000000000005</c:v>
+                  <c:v>541.31999999999994</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>547.56000000000006</c:v>
+                  <c:v>592.02</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>634.3599999999999</c:v>
+                  <c:v>662.72</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>731.16000000000008</c:v>
+                  <c:v>763.42000000000007</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>827.95999999999992</c:v>
+                  <c:v>864.12</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>924.76</c:v>
+                  <c:v>964.82</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>1021.5600000000001</c:v>
+                  <c:v>1065.5200000000002</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>1118.3599999999999</c:v>
+                  <c:v>1166.22</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>1215.1600000000001</c:v>
+                  <c:v>1266.92</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>1311.96</c:v>
+                  <c:v>1367.62</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>1408.76</c:v>
+                  <c:v>1468.3200000000002</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3984,58 +4181,58 @@
                   <c:v>190</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>264.48</c:v>
+                  <c:v>279.58499999999998</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>336.68000000000006</c:v>
+                  <c:v>356.53499999999997</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>408.88</c:v>
+                  <c:v>433.48500000000001</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>481.08</c:v>
+                  <c:v>510.43499999999995</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>553.28</c:v>
+                  <c:v>587.38499999999999</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>625.48</c:v>
+                  <c:v>664.33500000000004</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>697.68000000000006</c:v>
+                  <c:v>741.28500000000008</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>769.88</c:v>
+                  <c:v>818.23500000000001</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>842.08</c:v>
+                  <c:v>895.18500000000006</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>949.28</c:v>
+                  <c:v>989.63499999999999</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>1108.98</c:v>
+                  <c:v>1154.085</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>1268.6799999999998</c:v>
+                  <c:v>1318.5349999999999</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>1428.38</c:v>
+                  <c:v>1482.9850000000001</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>1588.0800000000002</c:v>
+                  <c:v>1647.4349999999999</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>1747.78</c:v>
+                  <c:v>1811.885</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>1907.48</c:v>
+                  <c:v>1976.335</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>2067.1800000000003</c:v>
+                  <c:v>2140.7849999999999</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>2226.88</c:v>
+                  <c:v>2305.2349999999997</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4152,58 +4349,58 @@
                   <c:v>250</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>360</c:v>
+                  <c:v>375</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>460</c:v>
+                  <c:v>480</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>560</c:v>
+                  <c:v>585</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>660</c:v>
+                  <c:v>690</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>760</c:v>
+                  <c:v>795</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>860</c:v>
+                  <c:v>900</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>960</c:v>
+                  <c:v>1005.0000000000001</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1060</c:v>
+                  <c:v>1110</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>1160</c:v>
+                  <c:v>1215</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>1260</c:v>
+                  <c:v>1320</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>1485</c:v>
+                  <c:v>1550</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>1710</c:v>
+                  <c:v>1779.9999999999998</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>1935</c:v>
+                  <c:v>2010</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>2160</c:v>
+                  <c:v>2240</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>2385</c:v>
+                  <c:v>2470</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>2610</c:v>
+                  <c:v>2700</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>2835</c:v>
+                  <c:v>2930</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>3060</c:v>
+                  <c:v>3160</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4320,58 +4517,58 @@
                   <c:v>310</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>462.52</c:v>
+                  <c:v>465</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>592.72</c:v>
+                  <c:v>603.88</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>722.92000000000007</c:v>
+                  <c:v>738.73</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>853.12000000000012</c:v>
+                  <c:v>873.57999999999993</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>983.31999999999994</c:v>
+                  <c:v>1008.43</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1113.5200000000002</c:v>
+                  <c:v>1143.2800000000002</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>1243.7200000000003</c:v>
+                  <c:v>1278.1300000000001</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1373.92</c:v>
+                  <c:v>1412.98</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>1504.1200000000003</c:v>
+                  <c:v>1547.83</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>1634.3200000000002</c:v>
+                  <c:v>1682.6799999999998</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>1862.0200000000002</c:v>
+                  <c:v>1947.5300000000002</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>2154.7199999999998</c:v>
+                  <c:v>2244.8799999999997</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>2447.42</c:v>
+                  <c:v>2542.23</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>2740.1200000000003</c:v>
+                  <c:v>2839.58</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>3032.82</c:v>
+                  <c:v>3136.93</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>3325.5200000000004</c:v>
+                  <c:v>3434.2799999999997</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>3618.2200000000003</c:v>
+                  <c:v>3731.6299999999997</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>3910.9200000000005</c:v>
+                  <c:v>4028.98</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4491,55 +4688,55 @@
                   <c:v>555</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>726.68</c:v>
+                  <c:v>728.9</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>889.48</c:v>
+                  <c:v>895.4</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1052.28</c:v>
+                  <c:v>1061.8999999999999</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1215.08</c:v>
+                  <c:v>1228.3999999999999</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1377.88</c:v>
+                  <c:v>1394.9</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>1540.68</c:v>
+                  <c:v>1561.4</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1703.4799999999998</c:v>
+                  <c:v>1727.8999999999999</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>1866.28</c:v>
+                  <c:v>1894.4</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>2029.0799999999997</c:v>
+                  <c:v>2060.8999999999996</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>2231.88</c:v>
+                  <c:v>2347.3999999999996</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>2594.6799999999994</c:v>
+                  <c:v>2713.8999999999996</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>2957.4799999999996</c:v>
+                  <c:v>3080.3999999999996</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>3320.28</c:v>
+                  <c:v>3446.9000000000005</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>3683.08</c:v>
+                  <c:v>3813.3999999999996</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>4045.88</c:v>
+                  <c:v>4179.8999999999996</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>4408.6799999999994</c:v>
+                  <c:v>4546.3999999999996</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>4771.4799999999996</c:v>
+                  <c:v>4912.8999999999996</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -6529,16 +6726,16 @@
       </c>
       <c r="F38" s="13">
         <f>INDEX(Parameters!$C$8:$G$8,1,MATCH($C38,Parameters!$C$6:$G$6,0))</f>
-        <v>0.09</v>
+        <v>0.12</v>
       </c>
       <c r="G38" s="13">
         <f>INDEX(Parameters!$C$9:$G$9,1,MATCH($C38,Parameters!$C$6:$G$6,0))</f>
-        <v>0.72</v>
+        <v>0.78</v>
       </c>
       <c r="H38" s="13"/>
       <c r="I38" s="14">
         <f>E38*G38</f>
-        <v>936</v>
+        <v>1014</v>
       </c>
       <c r="J38" s="14">
         <f>INDEX(Parameters!$C$10:$G$10,1,MATCH($D38,Parameters!$C$6:$G$6,0))</f>
@@ -6550,7 +6747,7 @@
       </c>
       <c r="L38" s="14">
         <f>I38+J38</f>
-        <v>3436</v>
+        <v>3514</v>
       </c>
       <c r="M38" s="1"/>
     </row>
@@ -6573,16 +6770,16 @@
       </c>
       <c r="F39" s="13">
         <f>INDEX(Parameters!$C$8:$G$8,1,MATCH($C39,Parameters!$C$6:$G$6,0))</f>
-        <v>0.105</v>
+        <v>0.13500000000000001</v>
       </c>
       <c r="G39" s="13">
         <f>INDEX(Parameters!$C$9:$G$9,1,MATCH($C39,Parameters!$C$6:$G$6,0))</f>
-        <v>0.76</v>
+        <v>0.81</v>
       </c>
       <c r="H39" s="13"/>
       <c r="I39" s="14">
         <f>E39*G39</f>
-        <v>1444</v>
+        <v>1539</v>
       </c>
       <c r="J39" s="14">
         <f>INDEX(Parameters!$C$10:$G$10,1,MATCH($D39,Parameters!$C$6:$G$6,0))</f>
@@ -6594,7 +6791,7 @@
       </c>
       <c r="L39" s="14">
         <f>I39+J39</f>
-        <v>3944</v>
+        <v>4039</v>
       </c>
       <c r="M39" s="1"/>
     </row>
@@ -6617,16 +6814,16 @@
       </c>
       <c r="F40" s="16">
         <f>INDEX(Parameters!$C$8:$G$8,1,MATCH($C40,Parameters!$C$6:$G$6,0))</f>
-        <v>0.12</v>
+        <v>0.15</v>
       </c>
       <c r="G40" s="16">
         <f>INDEX(Parameters!$C$9:$G$9,1,MATCH($C40,Parameters!$C$6:$G$6,0))</f>
-        <v>0.8</v>
+        <v>0.84</v>
       </c>
       <c r="H40" s="16"/>
       <c r="I40" s="17">
         <f>E40*G40</f>
-        <v>2000</v>
+        <v>2100</v>
       </c>
       <c r="J40" s="17">
         <f>INDEX(Parameters!$C$10:$G$10,1,MATCH($D40,Parameters!$C$6:$G$6,0))</f>
@@ -6638,7 +6835,7 @@
       </c>
       <c r="L40" s="17">
         <f>I40+J40</f>
-        <v>4500</v>
+        <v>4600</v>
       </c>
       <c r="M40" s="1"/>
     </row>
@@ -6661,16 +6858,16 @@
       </c>
       <c r="F41" s="13">
         <f>INDEX(Parameters!$C$8:$G$8,1,MATCH($C41,Parameters!$C$6:$G$6,0))</f>
-        <v>0.14500000000000002</v>
+        <v>0.16</v>
       </c>
       <c r="G41" s="13">
         <f>INDEX(Parameters!$C$9:$G$9,1,MATCH($C41,Parameters!$C$6:$G$6,0))</f>
-        <v>0.84000000000000008</v>
+        <v>0.87</v>
       </c>
       <c r="H41" s="13"/>
       <c r="I41" s="14">
         <f>E41*G41</f>
-        <v>2604.0000000000005</v>
+        <v>2697</v>
       </c>
       <c r="J41" s="14">
         <f>INDEX(Parameters!$C$10:$G$10,1,MATCH($D41,Parameters!$C$6:$G$6,0))</f>
@@ -6682,7 +6879,7 @@
       </c>
       <c r="L41" s="14">
         <f>I41+J41</f>
-        <v>5104</v>
+        <v>5197</v>
       </c>
       <c r="M41" s="1"/>
     </row>
@@ -6709,12 +6906,12 @@
       </c>
       <c r="G42" s="13">
         <f>INDEX(Parameters!$C$9:$G$9,1,MATCH($C42,Parameters!$C$6:$G$6,0))</f>
-        <v>0.88</v>
+        <v>0.9</v>
       </c>
       <c r="H42" s="13"/>
       <c r="I42" s="14">
         <f>E42*G42</f>
-        <v>3256</v>
+        <v>3330</v>
       </c>
       <c r="J42" s="14">
         <f>INDEX(Parameters!$C$10:$G$10,1,MATCH($D42,Parameters!$C$6:$G$6,0))</f>
@@ -6726,7 +6923,7 @@
       </c>
       <c r="L42" s="14">
         <f>I42+J42</f>
-        <v>5756</v>
+        <v>5830</v>
       </c>
       <c r="M42" s="1"/>
     </row>
@@ -6892,7 +7089,7 @@
       </c>
       <c r="C51" s="14">
         <f t="shared" si="0"/>
-        <v>126.36000000000001</v>
+        <v>130</v>
       </c>
       <c r="D51" s="14">
         <f t="shared" si="1"/>
@@ -6919,19 +7116,19 @@
       </c>
       <c r="C52" s="14">
         <f t="shared" si="0"/>
-        <v>173.16</v>
+        <v>186.42</v>
       </c>
       <c r="D52" s="14">
         <f t="shared" si="1"/>
-        <v>264.48</v>
+        <v>279.58499999999998</v>
       </c>
       <c r="E52" s="14">
         <f t="shared" si="2"/>
-        <v>360</v>
+        <v>375</v>
       </c>
       <c r="F52" s="14">
         <f t="shared" si="3"/>
-        <v>462.52</v>
+        <v>465</v>
       </c>
       <c r="G52" s="14">
         <f t="shared" si="4"/>
@@ -6946,23 +7143,23 @@
       </c>
       <c r="C53" s="14">
         <f t="shared" si="0"/>
-        <v>219.96</v>
+        <v>237.12</v>
       </c>
       <c r="D53" s="14">
         <f t="shared" si="1"/>
-        <v>336.68000000000006</v>
+        <v>356.53499999999997</v>
       </c>
       <c r="E53" s="14">
         <f t="shared" si="2"/>
-        <v>460</v>
+        <v>480</v>
       </c>
       <c r="F53" s="14">
         <f t="shared" si="3"/>
-        <v>592.72</v>
+        <v>603.88</v>
       </c>
       <c r="G53" s="14">
         <f t="shared" si="4"/>
-        <v>726.68</v>
+        <v>728.9</v>
       </c>
       <c r="M53" s="1"/>
     </row>
@@ -6973,23 +7170,23 @@
       </c>
       <c r="C54" s="14">
         <f t="shared" si="0"/>
-        <v>266.76</v>
+        <v>287.82</v>
       </c>
       <c r="D54" s="14">
         <f t="shared" si="1"/>
-        <v>408.88</v>
+        <v>433.48500000000001</v>
       </c>
       <c r="E54" s="14">
         <f t="shared" si="2"/>
-        <v>560</v>
+        <v>585</v>
       </c>
       <c r="F54" s="14">
         <f t="shared" si="3"/>
-        <v>722.92000000000007</v>
+        <v>738.73</v>
       </c>
       <c r="G54" s="14">
         <f t="shared" si="4"/>
-        <v>889.48</v>
+        <v>895.4</v>
       </c>
       <c r="M54" s="1"/>
     </row>
@@ -7000,23 +7197,23 @@
       </c>
       <c r="C55" s="14">
         <f t="shared" si="0"/>
-        <v>313.56</v>
+        <v>338.52</v>
       </c>
       <c r="D55" s="14">
         <f t="shared" si="1"/>
-        <v>481.08</v>
+        <v>510.43499999999995</v>
       </c>
       <c r="E55" s="14">
         <f t="shared" si="2"/>
-        <v>660</v>
+        <v>690</v>
       </c>
       <c r="F55" s="14">
         <f t="shared" si="3"/>
-        <v>853.12000000000012</v>
+        <v>873.57999999999993</v>
       </c>
       <c r="G55" s="14">
         <f t="shared" si="4"/>
-        <v>1052.28</v>
+        <v>1061.8999999999999</v>
       </c>
       <c r="M55" s="1"/>
     </row>
@@ -7027,23 +7224,23 @@
       </c>
       <c r="C56" s="14">
         <f t="shared" si="0"/>
-        <v>360.36</v>
+        <v>389.21999999999997</v>
       </c>
       <c r="D56" s="14">
         <f t="shared" si="1"/>
-        <v>553.28</v>
+        <v>587.38499999999999</v>
       </c>
       <c r="E56" s="14">
         <f t="shared" si="2"/>
-        <v>760</v>
+        <v>795</v>
       </c>
       <c r="F56" s="14">
         <f t="shared" si="3"/>
-        <v>983.31999999999994</v>
+        <v>1008.43</v>
       </c>
       <c r="G56" s="14">
         <f t="shared" si="4"/>
-        <v>1215.08</v>
+        <v>1228.3999999999999</v>
       </c>
       <c r="M56" s="1"/>
     </row>
@@ -7054,23 +7251,23 @@
       </c>
       <c r="C57" s="14">
         <f t="shared" si="0"/>
-        <v>407.16</v>
+        <v>439.92</v>
       </c>
       <c r="D57" s="14">
         <f t="shared" si="1"/>
-        <v>625.48</v>
+        <v>664.33500000000004</v>
       </c>
       <c r="E57" s="14">
         <f t="shared" si="2"/>
-        <v>860</v>
+        <v>900</v>
       </c>
       <c r="F57" s="14">
         <f t="shared" si="3"/>
-        <v>1113.5200000000002</v>
+        <v>1143.2800000000002</v>
       </c>
       <c r="G57" s="14">
         <f t="shared" si="4"/>
-        <v>1377.88</v>
+        <v>1394.9</v>
       </c>
       <c r="M57" s="1"/>
     </row>
@@ -7081,23 +7278,23 @@
       </c>
       <c r="C58" s="14">
         <f t="shared" si="0"/>
-        <v>453.96</v>
+        <v>490.62</v>
       </c>
       <c r="D58" s="14">
         <f t="shared" si="1"/>
-        <v>697.68000000000006</v>
+        <v>741.28500000000008</v>
       </c>
       <c r="E58" s="14">
         <f t="shared" si="2"/>
-        <v>960</v>
+        <v>1005.0000000000001</v>
       </c>
       <c r="F58" s="14">
         <f t="shared" si="3"/>
-        <v>1243.7200000000003</v>
+        <v>1278.1300000000001</v>
       </c>
       <c r="G58" s="14">
         <f t="shared" si="4"/>
-        <v>1540.68</v>
+        <v>1561.4</v>
       </c>
       <c r="M58" s="1"/>
     </row>
@@ -7108,23 +7305,23 @@
       </c>
       <c r="C59" s="14">
         <f t="shared" si="0"/>
-        <v>500.76000000000005</v>
+        <v>541.31999999999994</v>
       </c>
       <c r="D59" s="14">
         <f t="shared" si="1"/>
-        <v>769.88</v>
+        <v>818.23500000000001</v>
       </c>
       <c r="E59" s="14">
         <f t="shared" si="2"/>
-        <v>1060</v>
+        <v>1110</v>
       </c>
       <c r="F59" s="14">
         <f t="shared" si="3"/>
-        <v>1373.92</v>
+        <v>1412.98</v>
       </c>
       <c r="G59" s="14">
         <f t="shared" si="4"/>
-        <v>1703.4799999999998</v>
+        <v>1727.8999999999999</v>
       </c>
       <c r="M59" s="1"/>
     </row>
@@ -7135,23 +7332,23 @@
       </c>
       <c r="C60" s="14">
         <f t="shared" si="0"/>
-        <v>547.56000000000006</v>
+        <v>592.02</v>
       </c>
       <c r="D60" s="14">
         <f t="shared" si="1"/>
-        <v>842.08</v>
+        <v>895.18500000000006</v>
       </c>
       <c r="E60" s="14">
         <f t="shared" si="2"/>
-        <v>1160</v>
+        <v>1215</v>
       </c>
       <c r="F60" s="14">
         <f t="shared" si="3"/>
-        <v>1504.1200000000003</v>
+        <v>1547.83</v>
       </c>
       <c r="G60" s="14">
         <f t="shared" si="4"/>
-        <v>1866.28</v>
+        <v>1894.4</v>
       </c>
       <c r="M60" s="1"/>
     </row>
@@ -7162,23 +7359,23 @@
       </c>
       <c r="C61" s="14">
         <f t="shared" si="0"/>
-        <v>594.36</v>
+        <v>642.72</v>
       </c>
       <c r="D61" s="14">
         <f t="shared" si="1"/>
-        <v>914.28</v>
+        <v>972.13499999999999</v>
       </c>
       <c r="E61" s="14">
         <f t="shared" si="2"/>
-        <v>1260</v>
+        <v>1320</v>
       </c>
       <c r="F61" s="14">
         <f t="shared" si="3"/>
-        <v>1634.3200000000002</v>
+        <v>1682.6799999999998</v>
       </c>
       <c r="G61" s="14">
         <f t="shared" si="4"/>
-        <v>2029.0799999999997</v>
+        <v>2060.8999999999996</v>
       </c>
       <c r="M61" s="1"/>
     </row>
@@ -7189,23 +7386,23 @@
       </c>
       <c r="C62" s="14">
         <f t="shared" si="0"/>
-        <v>766.1600000000002</v>
+        <v>818.42000000000019</v>
       </c>
       <c r="D62" s="14">
         <f t="shared" si="1"/>
-        <v>1111.48</v>
+        <v>1174.085</v>
       </c>
       <c r="E62" s="14">
         <f t="shared" si="2"/>
-        <v>1485</v>
+        <v>1550</v>
       </c>
       <c r="F62" s="14">
         <f t="shared" si="3"/>
-        <v>1889.5200000000004</v>
+        <v>1942.5300000000002</v>
       </c>
       <c r="G62" s="14">
         <f t="shared" si="4"/>
-        <v>2316.88</v>
+        <v>2352.3999999999996</v>
       </c>
       <c r="M62" s="1"/>
     </row>
@@ -7216,23 +7413,23 @@
       </c>
       <c r="C63" s="14">
         <f t="shared" si="0"/>
-        <v>937.96</v>
+        <v>994.11999999999989</v>
       </c>
       <c r="D63" s="14">
         <f t="shared" si="1"/>
-        <v>1308.6799999999998</v>
+        <v>1376.0349999999999</v>
       </c>
       <c r="E63" s="14">
         <f t="shared" si="2"/>
-        <v>1710</v>
+        <v>1779.9999999999998</v>
       </c>
       <c r="F63" s="14">
         <f t="shared" si="3"/>
-        <v>2144.7199999999998</v>
+        <v>2202.3799999999997</v>
       </c>
       <c r="G63" s="14">
         <f t="shared" si="4"/>
-        <v>2604.6799999999998</v>
+        <v>2643.8999999999996</v>
       </c>
       <c r="M63" s="1"/>
     </row>
@@ -7243,23 +7440,23 @@
       </c>
       <c r="C64" s="14">
         <f t="shared" si="0"/>
-        <v>1109.76</v>
+        <v>1169.8200000000002</v>
       </c>
       <c r="D64" s="14">
         <f t="shared" si="1"/>
-        <v>1505.88</v>
+        <v>1577.9850000000001</v>
       </c>
       <c r="E64" s="14">
         <f t="shared" si="2"/>
-        <v>1935</v>
+        <v>2010</v>
       </c>
       <c r="F64" s="14">
         <f t="shared" si="3"/>
-        <v>2399.9200000000005</v>
+        <v>2462.23</v>
       </c>
       <c r="G64" s="14">
         <f t="shared" si="4"/>
-        <v>2892.4799999999996</v>
+        <v>2935.3999999999996</v>
       </c>
       <c r="M64" s="1"/>
     </row>
@@ -7270,23 +7467,23 @@
       </c>
       <c r="C65" s="14">
         <f t="shared" si="0"/>
-        <v>1281.5600000000002</v>
+        <v>1345.5200000000002</v>
       </c>
       <c r="D65" s="14">
         <f t="shared" si="1"/>
-        <v>1703.0800000000002</v>
+        <v>1779.9350000000002</v>
       </c>
       <c r="E65" s="14">
         <f t="shared" si="2"/>
-        <v>2160</v>
+        <v>2240</v>
       </c>
       <c r="F65" s="14">
         <f t="shared" si="3"/>
-        <v>2655.1200000000003</v>
+        <v>2722.08</v>
       </c>
       <c r="G65" s="14">
         <f t="shared" si="4"/>
-        <v>3180.28</v>
+        <v>3226.9</v>
       </c>
       <c r="M65" s="1"/>
     </row>
@@ -7297,23 +7494,23 @@
       </c>
       <c r="C66" s="14">
         <f t="shared" si="0"/>
-        <v>1453.3600000000001</v>
+        <v>1521.22</v>
       </c>
       <c r="D66" s="14">
         <f t="shared" si="1"/>
-        <v>1900.28</v>
+        <v>1981.885</v>
       </c>
       <c r="E66" s="14">
         <f t="shared" si="2"/>
-        <v>2385</v>
+        <v>2470</v>
       </c>
       <c r="F66" s="14">
         <f t="shared" si="3"/>
-        <v>2910.32</v>
+        <v>2981.93</v>
       </c>
       <c r="G66" s="14">
         <f t="shared" si="4"/>
-        <v>3468.08</v>
+        <v>3518.3999999999996</v>
       </c>
       <c r="M66" s="1"/>
     </row>
@@ -7324,23 +7521,23 @@
       </c>
       <c r="C67" s="14">
         <f t="shared" si="0"/>
-        <v>1625.1600000000003</v>
+        <v>1696.92</v>
       </c>
       <c r="D67" s="14">
         <f t="shared" si="1"/>
-        <v>2097.48</v>
+        <v>2183.835</v>
       </c>
       <c r="E67" s="14">
         <f t="shared" si="2"/>
-        <v>2610</v>
+        <v>2700</v>
       </c>
       <c r="F67" s="14">
         <f t="shared" si="3"/>
-        <v>3165.5200000000004</v>
+        <v>3241.7799999999997</v>
       </c>
       <c r="G67" s="14">
         <f t="shared" si="4"/>
-        <v>3755.88</v>
+        <v>3809.9</v>
       </c>
       <c r="M67" s="1"/>
     </row>
@@ -7351,23 +7548,23 @@
       </c>
       <c r="C68" s="14">
         <f t="shared" si="0"/>
-        <v>1796.96</v>
+        <v>1872.62</v>
       </c>
       <c r="D68" s="14">
         <f t="shared" si="1"/>
-        <v>2294.6800000000003</v>
+        <v>2385.7849999999999</v>
       </c>
       <c r="E68" s="14">
         <f t="shared" si="2"/>
-        <v>2835</v>
+        <v>2930</v>
       </c>
       <c r="F68" s="14">
         <f t="shared" si="3"/>
-        <v>3420.7200000000003</v>
+        <v>3501.6299999999997</v>
       </c>
       <c r="G68" s="14">
         <f t="shared" si="4"/>
-        <v>4043.68</v>
+        <v>4101.3999999999996</v>
       </c>
       <c r="M68" s="1"/>
     </row>
@@ -7378,23 +7575,23 @@
       </c>
       <c r="C69" s="14">
         <f t="shared" si="0"/>
-        <v>1968.76</v>
+        <v>2048.3200000000002</v>
       </c>
       <c r="D69" s="14">
         <f t="shared" si="1"/>
-        <v>2491.88</v>
+        <v>2587.7349999999997</v>
       </c>
       <c r="E69" s="14">
         <f t="shared" si="2"/>
-        <v>3060</v>
+        <v>3160</v>
       </c>
       <c r="F69" s="14">
         <f t="shared" si="3"/>
-        <v>3675.9200000000005</v>
+        <v>3761.48</v>
       </c>
       <c r="G69" s="14">
         <f t="shared" si="4"/>
-        <v>4331.4799999999996</v>
+        <v>4392.8999999999996</v>
       </c>
       <c r="M69" s="1"/>
     </row>
@@ -7402,19 +7599,19 @@
       <c r="A70" s="1"/>
       <c r="C70">
         <f t="shared" si="0"/>
-        <v>117</v>
+        <v>156</v>
       </c>
       <c r="D70">
         <f t="shared" si="1"/>
-        <v>199.5</v>
+        <v>256.5</v>
       </c>
       <c r="E70">
         <f t="shared" si="2"/>
-        <v>300</v>
+        <v>375</v>
       </c>
       <c r="F70">
         <f t="shared" si="3"/>
-        <v>449.50000000000006</v>
+        <v>496</v>
       </c>
       <c r="G70">
         <f t="shared" si="4"/>
@@ -7426,19 +7623,19 @@
       <c r="A71" s="1"/>
       <c r="C71">
         <f t="shared" si="0"/>
-        <v>117</v>
+        <v>156</v>
       </c>
       <c r="D71">
         <f t="shared" si="1"/>
-        <v>199.5</v>
+        <v>256.5</v>
       </c>
       <c r="E71">
         <f t="shared" si="2"/>
-        <v>300</v>
+        <v>375</v>
       </c>
       <c r="F71">
         <f t="shared" si="3"/>
-        <v>449.50000000000006</v>
+        <v>496</v>
       </c>
       <c r="G71">
         <f t="shared" si="4"/>
@@ -7450,19 +7647,19 @@
       <c r="A72" s="1"/>
       <c r="C72">
         <f t="shared" si="0"/>
-        <v>117</v>
+        <v>156</v>
       </c>
       <c r="D72">
         <f t="shared" si="1"/>
-        <v>199.5</v>
+        <v>256.5</v>
       </c>
       <c r="E72">
         <f t="shared" si="2"/>
-        <v>300</v>
+        <v>375</v>
       </c>
       <c r="F72">
         <f t="shared" si="3"/>
-        <v>449.50000000000006</v>
+        <v>496</v>
       </c>
       <c r="G72">
         <f t="shared" si="4"/>
@@ -7474,19 +7671,19 @@
       <c r="A73" s="1"/>
       <c r="C73">
         <f t="shared" si="0"/>
-        <v>117</v>
+        <v>156</v>
       </c>
       <c r="D73">
         <f t="shared" si="1"/>
-        <v>199.5</v>
+        <v>256.5</v>
       </c>
       <c r="E73">
         <f t="shared" si="2"/>
-        <v>300</v>
+        <v>375</v>
       </c>
       <c r="F73">
         <f t="shared" si="3"/>
-        <v>449.50000000000006</v>
+        <v>496</v>
       </c>
       <c r="G73">
         <f t="shared" si="4"/>
@@ -8128,16 +8325,16 @@
       </c>
       <c r="F38" s="13">
         <f>INDEX(Parameters!$C$8:$G$8,1,MATCH($C38,Parameters!$C$6:$G$6,0))</f>
-        <v>0.12</v>
+        <v>0.15</v>
       </c>
       <c r="G38" s="13">
         <f>INDEX(Parameters!$C$9:$G$9,1,MATCH($C38,Parameters!$C$6:$G$6,0))</f>
-        <v>0.8</v>
+        <v>0.84</v>
       </c>
       <c r="H38" s="13"/>
       <c r="I38" s="14">
         <f>E38*G38</f>
-        <v>2000</v>
+        <v>2100</v>
       </c>
       <c r="J38" s="14">
         <f>INDEX(Parameters!$C$10:$G$10,1,MATCH($D38,Parameters!$C$6:$G$6,0))</f>
@@ -8145,11 +8342,11 @@
       </c>
       <c r="K38" s="13">
         <f>INDEX(Parameters!$C$11:$G$11,1,MATCH($D38,Parameters!$C$6:$G$6,0))</f>
-        <v>0.56000000000000005</v>
+        <v>0.57999999999999996</v>
       </c>
       <c r="L38" s="14">
         <f>I38+J38</f>
-        <v>3000</v>
+        <v>3100</v>
       </c>
       <c r="M38" s="1"/>
     </row>
@@ -8172,16 +8369,16 @@
       </c>
       <c r="F39" s="13">
         <f>INDEX(Parameters!$C$8:$G$8,1,MATCH($C39,Parameters!$C$6:$G$6,0))</f>
-        <v>0.12</v>
+        <v>0.15</v>
       </c>
       <c r="G39" s="13">
         <f>INDEX(Parameters!$C$9:$G$9,1,MATCH($C39,Parameters!$C$6:$G$6,0))</f>
-        <v>0.8</v>
+        <v>0.84</v>
       </c>
       <c r="H39" s="13"/>
       <c r="I39" s="14">
         <f>E39*G39</f>
-        <v>2000</v>
+        <v>2100</v>
       </c>
       <c r="J39" s="14">
         <f>INDEX(Parameters!$C$10:$G$10,1,MATCH($D39,Parameters!$C$6:$G$6,0))</f>
@@ -8189,11 +8386,11 @@
       </c>
       <c r="K39" s="13">
         <f>INDEX(Parameters!$C$11:$G$11,1,MATCH($D39,Parameters!$C$6:$G$6,0))</f>
-        <v>0.57999999999999996</v>
+        <v>0.59</v>
       </c>
       <c r="L39" s="14">
         <f>I39+J39</f>
-        <v>3750</v>
+        <v>3850</v>
       </c>
       <c r="M39" s="1"/>
     </row>
@@ -8216,16 +8413,16 @@
       </c>
       <c r="F40" s="16">
         <f>INDEX(Parameters!$C$8:$G$8,1,MATCH($C40,Parameters!$C$6:$G$6,0))</f>
-        <v>0.12</v>
+        <v>0.15</v>
       </c>
       <c r="G40" s="16">
         <f>INDEX(Parameters!$C$9:$G$9,1,MATCH($C40,Parameters!$C$6:$G$6,0))</f>
-        <v>0.8</v>
+        <v>0.84</v>
       </c>
       <c r="H40" s="16"/>
       <c r="I40" s="17">
         <f>E40*G40</f>
-        <v>2000</v>
+        <v>2100</v>
       </c>
       <c r="J40" s="17">
         <f>INDEX(Parameters!$C$10:$G$10,1,MATCH($D40,Parameters!$C$6:$G$6,0))</f>
@@ -8237,7 +8434,7 @@
       </c>
       <c r="L40" s="17">
         <f>I40+J40</f>
-        <v>4500</v>
+        <v>4600</v>
       </c>
       <c r="M40" s="1"/>
     </row>
@@ -8260,16 +8457,16 @@
       </c>
       <c r="F41" s="13">
         <f>INDEX(Parameters!$C$8:$G$8,1,MATCH($C41,Parameters!$C$6:$G$6,0))</f>
-        <v>0.12</v>
+        <v>0.15</v>
       </c>
       <c r="G41" s="13">
         <f>INDEX(Parameters!$C$9:$G$9,1,MATCH($C41,Parameters!$C$6:$G$6,0))</f>
-        <v>0.8</v>
+        <v>0.84</v>
       </c>
       <c r="H41" s="13"/>
       <c r="I41" s="14">
         <f>E41*G41</f>
-        <v>2000</v>
+        <v>2100</v>
       </c>
       <c r="J41" s="14">
         <f>INDEX(Parameters!$C$10:$G$10,1,MATCH($D41,Parameters!$C$6:$G$6,0))</f>
@@ -8277,11 +8474,11 @@
       </c>
       <c r="K41" s="13">
         <f>INDEX(Parameters!$C$11:$G$11,1,MATCH($D41,Parameters!$C$6:$G$6,0))</f>
-        <v>0.62</v>
+        <v>0.61</v>
       </c>
       <c r="L41" s="14">
         <f>I41+J41</f>
-        <v>5250</v>
+        <v>5350</v>
       </c>
       <c r="M41" s="1"/>
     </row>
@@ -8304,16 +8501,16 @@
       </c>
       <c r="F42" s="13">
         <f>INDEX(Parameters!$C$8:$G$8,1,MATCH($C42,Parameters!$C$6:$G$6,0))</f>
-        <v>0.12</v>
+        <v>0.15</v>
       </c>
       <c r="G42" s="13">
         <f>INDEX(Parameters!$C$9:$G$9,1,MATCH($C42,Parameters!$C$6:$G$6,0))</f>
-        <v>0.8</v>
+        <v>0.84</v>
       </c>
       <c r="H42" s="13"/>
       <c r="I42" s="14">
         <f>E42*G42</f>
-        <v>2000</v>
+        <v>2100</v>
       </c>
       <c r="J42" s="14">
         <f>INDEX(Parameters!$C$10:$G$10,1,MATCH($D42,Parameters!$C$6:$G$6,0))</f>
@@ -8321,11 +8518,11 @@
       </c>
       <c r="K42" s="13">
         <f>INDEX(Parameters!$C$11:$G$11,1,MATCH($D42,Parameters!$C$6:$G$6,0))</f>
-        <v>0.64</v>
+        <v>0.62</v>
       </c>
       <c r="L42" s="14">
         <f>I42+J42</f>
-        <v>6000</v>
+        <v>6100</v>
       </c>
       <c r="M42" s="1"/>
     </row>
@@ -8518,23 +8715,23 @@
       </c>
       <c r="C52" s="14">
         <f t="shared" si="0"/>
-        <v>360</v>
+        <v>375</v>
       </c>
       <c r="D52" s="14">
         <f t="shared" si="1"/>
-        <v>360</v>
+        <v>375</v>
       </c>
       <c r="E52" s="14">
         <f t="shared" si="2"/>
-        <v>360</v>
+        <v>375</v>
       </c>
       <c r="F52" s="14">
         <f t="shared" si="3"/>
-        <v>360</v>
+        <v>375</v>
       </c>
       <c r="G52" s="14">
         <f t="shared" si="4"/>
-        <v>360</v>
+        <v>375</v>
       </c>
       <c r="M52" s="1"/>
     </row>
@@ -8545,23 +8742,23 @@
       </c>
       <c r="C53" s="14">
         <f t="shared" si="0"/>
-        <v>460</v>
+        <v>480</v>
       </c>
       <c r="D53" s="14">
         <f t="shared" si="1"/>
-        <v>460</v>
+        <v>480</v>
       </c>
       <c r="E53" s="14">
         <f t="shared" si="2"/>
-        <v>460</v>
+        <v>480</v>
       </c>
       <c r="F53" s="14">
         <f t="shared" si="3"/>
-        <v>460</v>
+        <v>480</v>
       </c>
       <c r="G53" s="14">
         <f t="shared" si="4"/>
-        <v>460</v>
+        <v>480</v>
       </c>
       <c r="M53" s="1"/>
     </row>
@@ -8572,23 +8769,23 @@
       </c>
       <c r="C54" s="14">
         <f t="shared" si="0"/>
-        <v>560</v>
+        <v>585</v>
       </c>
       <c r="D54" s="14">
         <f t="shared" si="1"/>
-        <v>560</v>
+        <v>585</v>
       </c>
       <c r="E54" s="14">
         <f t="shared" si="2"/>
-        <v>560</v>
+        <v>585</v>
       </c>
       <c r="F54" s="14">
         <f t="shared" si="3"/>
-        <v>560</v>
+        <v>585</v>
       </c>
       <c r="G54" s="14">
         <f t="shared" si="4"/>
-        <v>560</v>
+        <v>585</v>
       </c>
       <c r="M54" s="1"/>
     </row>
@@ -8599,23 +8796,23 @@
       </c>
       <c r="C55" s="14">
         <f t="shared" si="0"/>
-        <v>660</v>
+        <v>690</v>
       </c>
       <c r="D55" s="14">
         <f t="shared" si="1"/>
-        <v>660</v>
+        <v>690</v>
       </c>
       <c r="E55" s="14">
         <f t="shared" si="2"/>
-        <v>660</v>
+        <v>690</v>
       </c>
       <c r="F55" s="14">
         <f t="shared" si="3"/>
-        <v>660</v>
+        <v>690</v>
       </c>
       <c r="G55" s="14">
         <f t="shared" si="4"/>
-        <v>660</v>
+        <v>690</v>
       </c>
       <c r="M55" s="1"/>
     </row>
@@ -8626,23 +8823,23 @@
       </c>
       <c r="C56" s="14">
         <f t="shared" si="0"/>
-        <v>760</v>
+        <v>795</v>
       </c>
       <c r="D56" s="14">
         <f t="shared" si="1"/>
-        <v>760</v>
+        <v>795</v>
       </c>
       <c r="E56" s="14">
         <f t="shared" si="2"/>
-        <v>760</v>
+        <v>795</v>
       </c>
       <c r="F56" s="14">
         <f t="shared" si="3"/>
-        <v>760</v>
+        <v>795</v>
       </c>
       <c r="G56" s="14">
         <f t="shared" si="4"/>
-        <v>760</v>
+        <v>795</v>
       </c>
       <c r="M56" s="1"/>
     </row>
@@ -8653,23 +8850,23 @@
       </c>
       <c r="C57" s="14">
         <f t="shared" si="0"/>
-        <v>860</v>
+        <v>900</v>
       </c>
       <c r="D57" s="14">
         <f t="shared" si="1"/>
-        <v>860</v>
+        <v>900</v>
       </c>
       <c r="E57" s="14">
         <f t="shared" si="2"/>
-        <v>860</v>
+        <v>900</v>
       </c>
       <c r="F57" s="14">
         <f t="shared" si="3"/>
-        <v>860</v>
+        <v>900</v>
       </c>
       <c r="G57" s="14">
         <f t="shared" si="4"/>
-        <v>860</v>
+        <v>900</v>
       </c>
       <c r="M57" s="1"/>
     </row>
@@ -8680,23 +8877,23 @@
       </c>
       <c r="C58" s="14">
         <f t="shared" si="0"/>
-        <v>960</v>
+        <v>1005.0000000000001</v>
       </c>
       <c r="D58" s="14">
         <f t="shared" si="1"/>
-        <v>960</v>
+        <v>1005.0000000000001</v>
       </c>
       <c r="E58" s="14">
         <f t="shared" si="2"/>
-        <v>960</v>
+        <v>1005.0000000000001</v>
       </c>
       <c r="F58" s="14">
         <f t="shared" si="3"/>
-        <v>960</v>
+        <v>1005.0000000000001</v>
       </c>
       <c r="G58" s="14">
         <f t="shared" si="4"/>
-        <v>960</v>
+        <v>1005.0000000000001</v>
       </c>
       <c r="M58" s="1"/>
     </row>
@@ -8707,23 +8904,23 @@
       </c>
       <c r="C59" s="14">
         <f t="shared" si="0"/>
-        <v>1060</v>
+        <v>1110</v>
       </c>
       <c r="D59" s="14">
         <f t="shared" si="1"/>
-        <v>1060</v>
+        <v>1110</v>
       </c>
       <c r="E59" s="14">
         <f t="shared" si="2"/>
-        <v>1060</v>
+        <v>1110</v>
       </c>
       <c r="F59" s="14">
         <f t="shared" si="3"/>
-        <v>1060</v>
+        <v>1110</v>
       </c>
       <c r="G59" s="14">
         <f t="shared" si="4"/>
-        <v>1060</v>
+        <v>1110</v>
       </c>
       <c r="M59" s="1"/>
     </row>
@@ -8734,23 +8931,23 @@
       </c>
       <c r="C60" s="14">
         <f t="shared" si="0"/>
-        <v>1160</v>
+        <v>1215</v>
       </c>
       <c r="D60" s="14">
         <f t="shared" si="1"/>
-        <v>1160</v>
+        <v>1215</v>
       </c>
       <c r="E60" s="14">
         <f t="shared" si="2"/>
-        <v>1160</v>
+        <v>1215</v>
       </c>
       <c r="F60" s="14">
         <f t="shared" si="3"/>
-        <v>1160</v>
+        <v>1215</v>
       </c>
       <c r="G60" s="14">
         <f t="shared" si="4"/>
-        <v>1160</v>
+        <v>1215</v>
       </c>
       <c r="M60" s="1"/>
     </row>
@@ -8761,23 +8958,23 @@
       </c>
       <c r="C61" s="14">
         <f t="shared" si="0"/>
-        <v>1300</v>
+        <v>1340</v>
       </c>
       <c r="D61" s="14">
         <f t="shared" si="1"/>
-        <v>1295</v>
+        <v>1337.5</v>
       </c>
       <c r="E61" s="14">
         <f t="shared" si="2"/>
-        <v>1260</v>
+        <v>1320</v>
       </c>
       <c r="F61" s="14">
         <f t="shared" si="3"/>
-        <v>1260</v>
+        <v>1320</v>
       </c>
       <c r="G61" s="14">
         <f t="shared" si="4"/>
-        <v>1260</v>
+        <v>1320</v>
       </c>
       <c r="M61" s="1"/>
     </row>
@@ -8788,23 +8985,23 @@
       </c>
       <c r="C62" s="14">
         <f t="shared" si="0"/>
-        <v>1450</v>
+        <v>1495</v>
       </c>
       <c r="D62" s="14">
         <f t="shared" si="1"/>
-        <v>1482.5</v>
+        <v>1530</v>
       </c>
       <c r="E62" s="14">
         <f t="shared" si="2"/>
-        <v>1485</v>
+        <v>1550</v>
       </c>
       <c r="F62" s="14">
         <f t="shared" si="3"/>
-        <v>1457.5</v>
+        <v>1555</v>
       </c>
       <c r="G62" s="14">
         <f t="shared" si="4"/>
-        <v>1400</v>
+        <v>1545</v>
       </c>
       <c r="M62" s="1"/>
     </row>
@@ -8815,23 +9012,23 @@
       </c>
       <c r="C63" s="14">
         <f t="shared" si="0"/>
-        <v>1600</v>
+        <v>1649.9999999999998</v>
       </c>
       <c r="D63" s="14">
         <f t="shared" si="1"/>
-        <v>1670</v>
+        <v>1722.4999999999998</v>
       </c>
       <c r="E63" s="14">
         <f t="shared" si="2"/>
-        <v>1710</v>
+        <v>1779.9999999999998</v>
       </c>
       <c r="F63" s="14">
         <f t="shared" si="3"/>
-        <v>1720</v>
+        <v>1822.4999999999995</v>
       </c>
       <c r="G63" s="14">
         <f t="shared" si="4"/>
-        <v>1699.9999999999998</v>
+        <v>1849.9999999999995</v>
       </c>
       <c r="M63" s="1"/>
     </row>
@@ -8842,23 +9039,23 @@
       </c>
       <c r="C64" s="14">
         <f t="shared" si="0"/>
-        <v>1750</v>
+        <v>1805</v>
       </c>
       <c r="D64" s="14">
         <f t="shared" si="1"/>
-        <v>1857.5</v>
+        <v>1915</v>
       </c>
       <c r="E64" s="14">
         <f t="shared" si="2"/>
-        <v>1935</v>
+        <v>2010</v>
       </c>
       <c r="F64" s="14">
         <f t="shared" si="3"/>
-        <v>1982.5</v>
+        <v>2090</v>
       </c>
       <c r="G64" s="14">
         <f t="shared" si="4"/>
-        <v>2000</v>
+        <v>2155</v>
       </c>
       <c r="M64" s="1"/>
     </row>
@@ -8869,23 +9066,23 @@
       </c>
       <c r="C65" s="14">
         <f t="shared" si="0"/>
-        <v>1900</v>
+        <v>1960</v>
       </c>
       <c r="D65" s="14">
         <f t="shared" si="1"/>
-        <v>2045.0000000000002</v>
+        <v>2107.5</v>
       </c>
       <c r="E65" s="14">
         <f t="shared" si="2"/>
-        <v>2160</v>
+        <v>2240</v>
       </c>
       <c r="F65" s="14">
         <f t="shared" si="3"/>
-        <v>2245</v>
+        <v>2357.5</v>
       </c>
       <c r="G65" s="14">
         <f t="shared" si="4"/>
-        <v>2300</v>
+        <v>2460</v>
       </c>
       <c r="M65" s="1"/>
     </row>
@@ -8896,23 +9093,23 @@
       </c>
       <c r="C66" s="14">
         <f t="shared" si="0"/>
-        <v>2050</v>
+        <v>2115</v>
       </c>
       <c r="D66" s="14">
         <f t="shared" si="1"/>
-        <v>2232.5</v>
+        <v>2300</v>
       </c>
       <c r="E66" s="14">
         <f t="shared" si="2"/>
-        <v>2385</v>
+        <v>2470</v>
       </c>
       <c r="F66" s="14">
         <f t="shared" si="3"/>
-        <v>2507.5</v>
+        <v>2625</v>
       </c>
       <c r="G66" s="14">
         <f t="shared" si="4"/>
-        <v>2600</v>
+        <v>2765</v>
       </c>
       <c r="M66" s="1"/>
     </row>
@@ -8923,23 +9120,23 @@
       </c>
       <c r="C67" s="14">
         <f t="shared" si="0"/>
-        <v>2200</v>
+        <v>2270</v>
       </c>
       <c r="D67" s="14">
         <f t="shared" si="1"/>
-        <v>2420</v>
+        <v>2492.5</v>
       </c>
       <c r="E67" s="14">
         <f t="shared" si="2"/>
-        <v>2610</v>
+        <v>2700</v>
       </c>
       <c r="F67" s="14">
         <f t="shared" si="3"/>
-        <v>2770</v>
+        <v>2892.5</v>
       </c>
       <c r="G67" s="14">
         <f t="shared" si="4"/>
-        <v>2900</v>
+        <v>3070</v>
       </c>
       <c r="M67" s="1"/>
     </row>
@@ -8950,23 +9147,23 @@
       </c>
       <c r="C68" s="14">
         <f t="shared" si="0"/>
-        <v>2350</v>
+        <v>2425</v>
       </c>
       <c r="D68" s="14">
         <f t="shared" si="1"/>
-        <v>2607.5</v>
+        <v>2685</v>
       </c>
       <c r="E68" s="14">
         <f t="shared" si="2"/>
-        <v>2835</v>
+        <v>2930</v>
       </c>
       <c r="F68" s="14">
         <f t="shared" si="3"/>
-        <v>3032.5</v>
+        <v>3160</v>
       </c>
       <c r="G68" s="14">
         <f t="shared" si="4"/>
-        <v>3200</v>
+        <v>3375</v>
       </c>
       <c r="M68" s="1"/>
     </row>
@@ -8977,23 +9174,23 @@
       </c>
       <c r="C69" s="14">
         <f t="shared" si="0"/>
-        <v>2500</v>
+        <v>2580</v>
       </c>
       <c r="D69" s="14">
         <f t="shared" si="1"/>
-        <v>2795</v>
+        <v>2877.5</v>
       </c>
       <c r="E69" s="14">
         <f t="shared" si="2"/>
-        <v>3060</v>
+        <v>3160</v>
       </c>
       <c r="F69" s="14">
         <f t="shared" si="3"/>
-        <v>3295</v>
+        <v>3427.5</v>
       </c>
       <c r="G69" s="14">
         <f t="shared" si="4"/>
-        <v>3500</v>
+        <v>3680</v>
       </c>
       <c r="M69" s="1"/>
     </row>
@@ -9001,23 +9198,23 @@
       <c r="A70" s="1"/>
       <c r="C70">
         <f t="shared" si="0"/>
-        <v>300</v>
+        <v>375</v>
       </c>
       <c r="D70">
         <f t="shared" si="1"/>
-        <v>300</v>
+        <v>375</v>
       </c>
       <c r="E70">
         <f t="shared" si="2"/>
-        <v>300</v>
+        <v>375</v>
       </c>
       <c r="F70">
         <f t="shared" si="3"/>
-        <v>300</v>
+        <v>375</v>
       </c>
       <c r="G70">
         <f t="shared" si="4"/>
-        <v>300</v>
+        <v>375</v>
       </c>
       <c r="M70" s="1"/>
     </row>
@@ -9025,23 +9222,23 @@
       <c r="A71" s="1"/>
       <c r="C71">
         <f t="shared" si="0"/>
-        <v>300</v>
+        <v>375</v>
       </c>
       <c r="D71">
         <f t="shared" si="1"/>
-        <v>300</v>
+        <v>375</v>
       </c>
       <c r="E71">
         <f t="shared" si="2"/>
-        <v>300</v>
+        <v>375</v>
       </c>
       <c r="F71">
         <f t="shared" si="3"/>
-        <v>300</v>
+        <v>375</v>
       </c>
       <c r="G71">
         <f t="shared" si="4"/>
-        <v>300</v>
+        <v>375</v>
       </c>
       <c r="M71" s="1"/>
     </row>
@@ -9049,23 +9246,23 @@
       <c r="A72" s="1"/>
       <c r="C72">
         <f t="shared" si="0"/>
-        <v>300</v>
+        <v>375</v>
       </c>
       <c r="D72">
         <f t="shared" si="1"/>
-        <v>300</v>
+        <v>375</v>
       </c>
       <c r="E72">
         <f t="shared" si="2"/>
-        <v>300</v>
+        <v>375</v>
       </c>
       <c r="F72">
         <f t="shared" si="3"/>
-        <v>300</v>
+        <v>375</v>
       </c>
       <c r="G72">
         <f t="shared" si="4"/>
-        <v>300</v>
+        <v>375</v>
       </c>
       <c r="M72" s="1"/>
     </row>
@@ -9073,23 +9270,23 @@
       <c r="A73" s="1"/>
       <c r="C73">
         <f t="shared" si="0"/>
-        <v>300</v>
+        <v>375</v>
       </c>
       <c r="D73">
         <f t="shared" si="1"/>
-        <v>300</v>
+        <v>375</v>
       </c>
       <c r="E73">
         <f t="shared" si="2"/>
-        <v>300</v>
+        <v>375</v>
       </c>
       <c r="F73">
         <f t="shared" si="3"/>
-        <v>300</v>
+        <v>375</v>
       </c>
       <c r="G73">
         <f t="shared" si="4"/>
-        <v>300</v>
+        <v>375</v>
       </c>
       <c r="M73" s="1"/>
     </row>
@@ -9163,7 +9360,7 @@
       <c r="A3" s="20"/>
       <c r="B3" s="28" t="str">
         <f>"Rally2 Gravel · "&amp;Parameters!E35&amp;"；单一回弹旋钮，LSR：−40 / −30 / −20 / −10 / 0"</f>
-        <v>Rally2 Gravel · Type-B；单一回弹旋钮，LSR：−40 / −30 / −20 / −10 / 0</v>
+        <v>Rally2 Gravel · Type-A；单一回弹旋钮，LSR：−40 / −30 / −20 / −10 / 0</v>
       </c>
       <c r="C3" s="20"/>
       <c r="D3" s="20"/>
@@ -11389,16 +11586,16 @@
       </c>
       <c r="F38" s="13">
         <f>INDEX(Parameters!$C$8:$G$8,1,MATCH($C38,Parameters!$C$6:$G$6,0))</f>
-        <v>0.09</v>
+        <v>0.12</v>
       </c>
       <c r="G38" s="13">
         <f>INDEX(Parameters!$C$9:$G$9,1,MATCH($C38,Parameters!$C$6:$G$6,0))</f>
-        <v>0.72</v>
+        <v>0.78</v>
       </c>
       <c r="H38" s="13"/>
       <c r="I38" s="14">
         <f>E38*G38</f>
-        <v>936</v>
+        <v>1014</v>
       </c>
       <c r="J38" s="14">
         <f>INDEX(Parameters!$C$10:$G$10,1,MATCH($D38,Parameters!$C$6:$G$6,0))</f>
@@ -11406,11 +11603,11 @@
       </c>
       <c r="K38" s="13">
         <f>INDEX(Parameters!$C$11:$G$11,1,MATCH($D38,Parameters!$C$6:$G$6,0))</f>
-        <v>0.56000000000000005</v>
+        <v>0.57999999999999996</v>
       </c>
       <c r="L38" s="14">
         <f>I38+J38</f>
-        <v>1936</v>
+        <v>2014</v>
       </c>
       <c r="M38" s="1"/>
     </row>
@@ -11433,16 +11630,16 @@
       </c>
       <c r="F39" s="13">
         <f>INDEX(Parameters!$C$8:$G$8,1,MATCH($C39,Parameters!$C$6:$G$6,0))</f>
-        <v>0.105</v>
+        <v>0.13500000000000001</v>
       </c>
       <c r="G39" s="13">
         <f>INDEX(Parameters!$C$9:$G$9,1,MATCH($C39,Parameters!$C$6:$G$6,0))</f>
-        <v>0.76</v>
+        <v>0.81</v>
       </c>
       <c r="H39" s="13"/>
       <c r="I39" s="14">
         <f>E39*G39</f>
-        <v>1444</v>
+        <v>1539</v>
       </c>
       <c r="J39" s="14">
         <f>INDEX(Parameters!$C$10:$G$10,1,MATCH($D39,Parameters!$C$6:$G$6,0))</f>
@@ -11450,11 +11647,11 @@
       </c>
       <c r="K39" s="13">
         <f>INDEX(Parameters!$C$11:$G$11,1,MATCH($D39,Parameters!$C$6:$G$6,0))</f>
-        <v>0.57999999999999996</v>
+        <v>0.59</v>
       </c>
       <c r="L39" s="14">
         <f>I39+J39</f>
-        <v>3194</v>
+        <v>3289</v>
       </c>
       <c r="M39" s="1"/>
     </row>
@@ -11477,16 +11674,16 @@
       </c>
       <c r="F40" s="16">
         <f>INDEX(Parameters!$C$8:$G$8,1,MATCH($C40,Parameters!$C$6:$G$6,0))</f>
-        <v>0.12</v>
+        <v>0.15</v>
       </c>
       <c r="G40" s="16">
         <f>INDEX(Parameters!$C$9:$G$9,1,MATCH($C40,Parameters!$C$6:$G$6,0))</f>
-        <v>0.8</v>
+        <v>0.84</v>
       </c>
       <c r="H40" s="16"/>
       <c r="I40" s="17">
         <f>E40*G40</f>
-        <v>2000</v>
+        <v>2100</v>
       </c>
       <c r="J40" s="17">
         <f>INDEX(Parameters!$C$10:$G$10,1,MATCH($D40,Parameters!$C$6:$G$6,0))</f>
@@ -11498,7 +11695,7 @@
       </c>
       <c r="L40" s="17">
         <f>I40+J40</f>
-        <v>4500</v>
+        <v>4600</v>
       </c>
       <c r="M40" s="1"/>
     </row>
@@ -11521,16 +11718,16 @@
       </c>
       <c r="F41" s="13">
         <f>INDEX(Parameters!$C$8:$G$8,1,MATCH($C41,Parameters!$C$6:$G$6,0))</f>
-        <v>0.14500000000000002</v>
+        <v>0.16</v>
       </c>
       <c r="G41" s="13">
         <f>INDEX(Parameters!$C$9:$G$9,1,MATCH($C41,Parameters!$C$6:$G$6,0))</f>
-        <v>0.84000000000000008</v>
+        <v>0.87</v>
       </c>
       <c r="H41" s="13"/>
       <c r="I41" s="14">
         <f>E41*G41</f>
-        <v>2604.0000000000005</v>
+        <v>2697</v>
       </c>
       <c r="J41" s="14">
         <f>INDEX(Parameters!$C$10:$G$10,1,MATCH($D41,Parameters!$C$6:$G$6,0))</f>
@@ -11538,11 +11735,11 @@
       </c>
       <c r="K41" s="13">
         <f>INDEX(Parameters!$C$11:$G$11,1,MATCH($D41,Parameters!$C$6:$G$6,0))</f>
-        <v>0.62</v>
+        <v>0.61</v>
       </c>
       <c r="L41" s="14">
         <f>I41+J41</f>
-        <v>5854</v>
+        <v>5947</v>
       </c>
       <c r="M41" s="1"/>
     </row>
@@ -11569,12 +11766,12 @@
       </c>
       <c r="G42" s="13">
         <f>INDEX(Parameters!$C$9:$G$9,1,MATCH($C42,Parameters!$C$6:$G$6,0))</f>
-        <v>0.88</v>
+        <v>0.9</v>
       </c>
       <c r="H42" s="13"/>
       <c r="I42" s="14">
         <f>E42*G42</f>
-        <v>3256</v>
+        <v>3330</v>
       </c>
       <c r="J42" s="14">
         <f>INDEX(Parameters!$C$10:$G$10,1,MATCH($D42,Parameters!$C$6:$G$6,0))</f>
@@ -11582,11 +11779,11 @@
       </c>
       <c r="K42" s="13">
         <f>INDEX(Parameters!$C$11:$G$11,1,MATCH($D42,Parameters!$C$6:$G$6,0))</f>
-        <v>0.64</v>
+        <v>0.62</v>
       </c>
       <c r="L42" s="14">
         <f>I42+J42</f>
-        <v>7256</v>
+        <v>7330</v>
       </c>
       <c r="M42" s="1"/>
     </row>
@@ -11812,7 +12009,7 @@
       </c>
       <c r="C51" s="14">
         <f t="shared" si="0"/>
-        <v>126.36000000000001</v>
+        <v>130</v>
       </c>
       <c r="D51" s="14">
         <f t="shared" si="1"/>
@@ -11859,19 +12056,19 @@
       </c>
       <c r="C52" s="14">
         <f t="shared" si="0"/>
-        <v>173.16</v>
+        <v>186.42</v>
       </c>
       <c r="D52" s="14">
         <f t="shared" si="1"/>
-        <v>264.48</v>
+        <v>279.58499999999998</v>
       </c>
       <c r="E52" s="14">
         <f t="shared" si="2"/>
-        <v>360</v>
+        <v>375</v>
       </c>
       <c r="F52" s="14">
         <f t="shared" si="3"/>
-        <v>462.52</v>
+        <v>465</v>
       </c>
       <c r="G52" s="14">
         <f t="shared" si="4"/>
@@ -11906,23 +12103,23 @@
       </c>
       <c r="C53" s="14">
         <f t="shared" si="0"/>
-        <v>219.96</v>
+        <v>237.12</v>
       </c>
       <c r="D53" s="14">
         <f t="shared" si="1"/>
-        <v>336.68000000000006</v>
+        <v>356.53499999999997</v>
       </c>
       <c r="E53" s="14">
         <f t="shared" si="2"/>
-        <v>460</v>
+        <v>480</v>
       </c>
       <c r="F53" s="14">
         <f t="shared" si="3"/>
-        <v>592.72</v>
+        <v>603.88</v>
       </c>
       <c r="G53" s="14">
         <f t="shared" si="4"/>
-        <v>726.68</v>
+        <v>728.9</v>
       </c>
       <c r="H53" s="1">
         <f>-'LSR Sweep'!C53</f>
@@ -11953,23 +12150,23 @@
       </c>
       <c r="C54" s="14">
         <f t="shared" si="0"/>
-        <v>266.76</v>
+        <v>287.82</v>
       </c>
       <c r="D54" s="14">
         <f t="shared" si="1"/>
-        <v>408.88</v>
+        <v>433.48500000000001</v>
       </c>
       <c r="E54" s="14">
         <f t="shared" si="2"/>
-        <v>560</v>
+        <v>585</v>
       </c>
       <c r="F54" s="14">
         <f t="shared" si="3"/>
-        <v>722.92000000000007</v>
+        <v>738.73</v>
       </c>
       <c r="G54" s="14">
         <f t="shared" si="4"/>
-        <v>889.48</v>
+        <v>895.4</v>
       </c>
       <c r="H54" s="1">
         <f>-'LSR Sweep'!C54</f>
@@ -12000,23 +12197,23 @@
       </c>
       <c r="C55" s="14">
         <f t="shared" si="0"/>
-        <v>313.56</v>
+        <v>338.52</v>
       </c>
       <c r="D55" s="14">
         <f t="shared" si="1"/>
-        <v>481.08</v>
+        <v>510.43499999999995</v>
       </c>
       <c r="E55" s="14">
         <f t="shared" si="2"/>
-        <v>660</v>
+        <v>690</v>
       </c>
       <c r="F55" s="14">
         <f t="shared" si="3"/>
-        <v>853.12000000000012</v>
+        <v>873.57999999999993</v>
       </c>
       <c r="G55" s="14">
         <f t="shared" si="4"/>
-        <v>1052.28</v>
+        <v>1061.8999999999999</v>
       </c>
       <c r="H55" s="1">
         <f>-'LSR Sweep'!C55</f>
@@ -12047,23 +12244,23 @@
       </c>
       <c r="C56" s="14">
         <f t="shared" si="0"/>
-        <v>360.36</v>
+        <v>389.21999999999997</v>
       </c>
       <c r="D56" s="14">
         <f t="shared" si="1"/>
-        <v>553.28</v>
+        <v>587.38499999999999</v>
       </c>
       <c r="E56" s="14">
         <f t="shared" si="2"/>
-        <v>760</v>
+        <v>795</v>
       </c>
       <c r="F56" s="14">
         <f t="shared" si="3"/>
-        <v>983.31999999999994</v>
+        <v>1008.43</v>
       </c>
       <c r="G56" s="14">
         <f t="shared" si="4"/>
-        <v>1215.08</v>
+        <v>1228.3999999999999</v>
       </c>
       <c r="H56" s="1">
         <f>-'LSR Sweep'!C56</f>
@@ -12094,23 +12291,23 @@
       </c>
       <c r="C57" s="14">
         <f t="shared" si="0"/>
-        <v>407.16</v>
+        <v>439.92</v>
       </c>
       <c r="D57" s="14">
         <f t="shared" si="1"/>
-        <v>625.48</v>
+        <v>664.33500000000004</v>
       </c>
       <c r="E57" s="14">
         <f t="shared" si="2"/>
-        <v>860</v>
+        <v>900</v>
       </c>
       <c r="F57" s="14">
         <f t="shared" si="3"/>
-        <v>1113.5200000000002</v>
+        <v>1143.2800000000002</v>
       </c>
       <c r="G57" s="14">
         <f t="shared" si="4"/>
-        <v>1377.88</v>
+        <v>1394.9</v>
       </c>
       <c r="H57" s="1">
         <f>-'LSR Sweep'!C57</f>
@@ -12141,23 +12338,23 @@
       </c>
       <c r="C58" s="14">
         <f t="shared" si="0"/>
-        <v>453.96</v>
+        <v>490.62</v>
       </c>
       <c r="D58" s="14">
         <f t="shared" si="1"/>
-        <v>697.68000000000006</v>
+        <v>741.28500000000008</v>
       </c>
       <c r="E58" s="14">
         <f t="shared" si="2"/>
-        <v>960</v>
+        <v>1005.0000000000001</v>
       </c>
       <c r="F58" s="14">
         <f t="shared" si="3"/>
-        <v>1243.7200000000003</v>
+        <v>1278.1300000000001</v>
       </c>
       <c r="G58" s="14">
         <f t="shared" si="4"/>
-        <v>1540.68</v>
+        <v>1561.4</v>
       </c>
       <c r="H58" s="1">
         <f>-'LSR Sweep'!C58</f>
@@ -12188,23 +12385,23 @@
       </c>
       <c r="C59" s="14">
         <f t="shared" si="0"/>
-        <v>500.76000000000005</v>
+        <v>541.31999999999994</v>
       </c>
       <c r="D59" s="14">
         <f t="shared" si="1"/>
-        <v>769.88</v>
+        <v>818.23500000000001</v>
       </c>
       <c r="E59" s="14">
         <f t="shared" si="2"/>
-        <v>1060</v>
+        <v>1110</v>
       </c>
       <c r="F59" s="14">
         <f t="shared" si="3"/>
-        <v>1373.92</v>
+        <v>1412.98</v>
       </c>
       <c r="G59" s="14">
         <f t="shared" si="4"/>
-        <v>1703.4799999999998</v>
+        <v>1727.8999999999999</v>
       </c>
       <c r="H59" s="1">
         <f>-'LSR Sweep'!C59</f>
@@ -12235,23 +12432,23 @@
       </c>
       <c r="C60" s="14">
         <f t="shared" si="0"/>
-        <v>547.56000000000006</v>
+        <v>592.02</v>
       </c>
       <c r="D60" s="14">
         <f t="shared" si="1"/>
-        <v>842.08</v>
+        <v>895.18500000000006</v>
       </c>
       <c r="E60" s="14">
         <f t="shared" si="2"/>
-        <v>1160</v>
+        <v>1215</v>
       </c>
       <c r="F60" s="14">
         <f t="shared" si="3"/>
-        <v>1504.1200000000003</v>
+        <v>1547.83</v>
       </c>
       <c r="G60" s="14">
         <f t="shared" si="4"/>
-        <v>1866.28</v>
+        <v>1894.4</v>
       </c>
       <c r="H60" s="1">
         <f>-'LSR Sweep'!C60</f>
@@ -12282,23 +12479,23 @@
       </c>
       <c r="C61" s="14">
         <f t="shared" si="0"/>
-        <v>634.3599999999999</v>
+        <v>662.72</v>
       </c>
       <c r="D61" s="14">
         <f t="shared" si="1"/>
-        <v>949.28</v>
+        <v>989.63499999999999</v>
       </c>
       <c r="E61" s="14">
         <f t="shared" si="2"/>
-        <v>1260</v>
+        <v>1320</v>
       </c>
       <c r="F61" s="14">
         <f t="shared" si="3"/>
-        <v>1634.3200000000002</v>
+        <v>1682.6799999999998</v>
       </c>
       <c r="G61" s="14">
         <f t="shared" si="4"/>
-        <v>2029.0799999999997</v>
+        <v>2060.8999999999996</v>
       </c>
       <c r="H61" s="1">
         <f>-'LSR Sweep'!C61</f>
@@ -12329,23 +12526,23 @@
       </c>
       <c r="C62" s="14">
         <f t="shared" si="0"/>
-        <v>731.16000000000008</v>
+        <v>763.42000000000007</v>
       </c>
       <c r="D62" s="14">
         <f t="shared" si="1"/>
-        <v>1108.98</v>
+        <v>1154.085</v>
       </c>
       <c r="E62" s="14">
         <f t="shared" si="2"/>
-        <v>1485</v>
+        <v>1550</v>
       </c>
       <c r="F62" s="14">
         <f t="shared" si="3"/>
-        <v>1862.0200000000002</v>
+        <v>1947.5300000000002</v>
       </c>
       <c r="G62" s="14">
         <f t="shared" si="4"/>
-        <v>2231.88</v>
+        <v>2347.3999999999996</v>
       </c>
       <c r="H62" s="1">
         <f>-'LSR Sweep'!C62</f>
@@ -12376,23 +12573,23 @@
       </c>
       <c r="C63" s="14">
         <f t="shared" si="0"/>
-        <v>827.95999999999992</v>
+        <v>864.12</v>
       </c>
       <c r="D63" s="14">
         <f t="shared" si="1"/>
-        <v>1268.6799999999998</v>
+        <v>1318.5349999999999</v>
       </c>
       <c r="E63" s="14">
         <f t="shared" si="2"/>
-        <v>1710</v>
+        <v>1779.9999999999998</v>
       </c>
       <c r="F63" s="14">
         <f t="shared" si="3"/>
-        <v>2154.7199999999998</v>
+        <v>2244.8799999999997</v>
       </c>
       <c r="G63" s="14">
         <f t="shared" si="4"/>
-        <v>2594.6799999999994</v>
+        <v>2713.8999999999996</v>
       </c>
       <c r="H63" s="1">
         <f>-'LSR Sweep'!C63</f>
@@ -12423,23 +12620,23 @@
       </c>
       <c r="C64" s="14">
         <f t="shared" si="0"/>
-        <v>924.76</v>
+        <v>964.82</v>
       </c>
       <c r="D64" s="14">
         <f t="shared" si="1"/>
-        <v>1428.38</v>
+        <v>1482.9850000000001</v>
       </c>
       <c r="E64" s="14">
         <f t="shared" si="2"/>
-        <v>1935</v>
+        <v>2010</v>
       </c>
       <c r="F64" s="14">
         <f t="shared" si="3"/>
-        <v>2447.42</v>
+        <v>2542.23</v>
       </c>
       <c r="G64" s="14">
         <f t="shared" si="4"/>
-        <v>2957.4799999999996</v>
+        <v>3080.3999999999996</v>
       </c>
       <c r="H64" s="1">
         <f>-'LSR Sweep'!C64</f>
@@ -12470,23 +12667,23 @@
       </c>
       <c r="C65" s="14">
         <f t="shared" si="0"/>
-        <v>1021.5600000000001</v>
+        <v>1065.5200000000002</v>
       </c>
       <c r="D65" s="14">
         <f t="shared" si="1"/>
-        <v>1588.0800000000002</v>
+        <v>1647.4349999999999</v>
       </c>
       <c r="E65" s="14">
         <f t="shared" si="2"/>
-        <v>2160</v>
+        <v>2240</v>
       </c>
       <c r="F65" s="14">
         <f t="shared" si="3"/>
-        <v>2740.1200000000003</v>
+        <v>2839.58</v>
       </c>
       <c r="G65" s="14">
         <f t="shared" si="4"/>
-        <v>3320.28</v>
+        <v>3446.9000000000005</v>
       </c>
       <c r="H65" s="1">
         <f>-'LSR Sweep'!C65</f>
@@ -12517,23 +12714,23 @@
       </c>
       <c r="C66" s="14">
         <f t="shared" si="0"/>
-        <v>1118.3599999999999</v>
+        <v>1166.22</v>
       </c>
       <c r="D66" s="14">
         <f t="shared" si="1"/>
-        <v>1747.78</v>
+        <v>1811.885</v>
       </c>
       <c r="E66" s="14">
         <f t="shared" si="2"/>
-        <v>2385</v>
+        <v>2470</v>
       </c>
       <c r="F66" s="14">
         <f t="shared" si="3"/>
-        <v>3032.82</v>
+        <v>3136.93</v>
       </c>
       <c r="G66" s="14">
         <f t="shared" si="4"/>
-        <v>3683.08</v>
+        <v>3813.3999999999996</v>
       </c>
       <c r="H66" s="1">
         <f>-'LSR Sweep'!C66</f>
@@ -12564,23 +12761,23 @@
       </c>
       <c r="C67" s="14">
         <f t="shared" si="0"/>
-        <v>1215.1600000000001</v>
+        <v>1266.92</v>
       </c>
       <c r="D67" s="14">
         <f t="shared" si="1"/>
-        <v>1907.48</v>
+        <v>1976.335</v>
       </c>
       <c r="E67" s="14">
         <f t="shared" si="2"/>
-        <v>2610</v>
+        <v>2700</v>
       </c>
       <c r="F67" s="14">
         <f t="shared" si="3"/>
-        <v>3325.5200000000004</v>
+        <v>3434.2799999999997</v>
       </c>
       <c r="G67" s="14">
         <f t="shared" si="4"/>
-        <v>4045.88</v>
+        <v>4179.8999999999996</v>
       </c>
       <c r="H67" s="1">
         <f>-'LSR Sweep'!C67</f>
@@ -12611,23 +12808,23 @@
       </c>
       <c r="C68" s="14">
         <f t="shared" si="0"/>
-        <v>1311.96</v>
+        <v>1367.62</v>
       </c>
       <c r="D68" s="14">
         <f t="shared" si="1"/>
-        <v>2067.1800000000003</v>
+        <v>2140.7849999999999</v>
       </c>
       <c r="E68" s="14">
         <f t="shared" si="2"/>
-        <v>2835</v>
+        <v>2930</v>
       </c>
       <c r="F68" s="14">
         <f t="shared" si="3"/>
-        <v>3618.2200000000003</v>
+        <v>3731.6299999999997</v>
       </c>
       <c r="G68" s="14">
         <f t="shared" si="4"/>
-        <v>4408.6799999999994</v>
+        <v>4546.3999999999996</v>
       </c>
       <c r="H68" s="1">
         <f>-'LSR Sweep'!C68</f>
@@ -12658,23 +12855,23 @@
       </c>
       <c r="C69" s="14">
         <f t="shared" si="0"/>
-        <v>1408.76</v>
+        <v>1468.3200000000002</v>
       </c>
       <c r="D69" s="14">
         <f t="shared" si="1"/>
-        <v>2226.88</v>
+        <v>2305.2349999999997</v>
       </c>
       <c r="E69" s="14">
         <f t="shared" si="2"/>
-        <v>3060</v>
+        <v>3160</v>
       </c>
       <c r="F69" s="14">
         <f t="shared" si="3"/>
-        <v>3910.9200000000005</v>
+        <v>4028.98</v>
       </c>
       <c r="G69" s="14">
         <f t="shared" si="4"/>
-        <v>4771.4799999999996</v>
+        <v>4912.8999999999996</v>
       </c>
       <c r="H69" s="1">
         <f>-'LSR Sweep'!C69</f>
@@ -12702,19 +12899,19 @@
       <c r="A70" s="1"/>
       <c r="C70">
         <f t="shared" si="0"/>
-        <v>117</v>
+        <v>156</v>
       </c>
       <c r="D70">
         <f t="shared" si="1"/>
-        <v>199.5</v>
+        <v>256.5</v>
       </c>
       <c r="E70">
         <f t="shared" si="2"/>
-        <v>300</v>
+        <v>375</v>
       </c>
       <c r="F70">
         <f t="shared" si="3"/>
-        <v>449.50000000000006</v>
+        <v>496</v>
       </c>
       <c r="G70">
         <f t="shared" si="4"/>
@@ -12726,19 +12923,19 @@
       <c r="A71" s="1"/>
       <c r="C71">
         <f t="shared" si="0"/>
-        <v>117</v>
+        <v>156</v>
       </c>
       <c r="D71">
         <f t="shared" si="1"/>
-        <v>199.5</v>
+        <v>256.5</v>
       </c>
       <c r="E71">
         <f t="shared" si="2"/>
-        <v>300</v>
+        <v>375</v>
       </c>
       <c r="F71">
         <f t="shared" si="3"/>
-        <v>449.50000000000006</v>
+        <v>496</v>
       </c>
       <c r="G71">
         <f t="shared" si="4"/>
@@ -12750,19 +12947,19 @@
       <c r="A72" s="1"/>
       <c r="C72">
         <f t="shared" si="0"/>
-        <v>117</v>
+        <v>156</v>
       </c>
       <c r="D72">
         <f t="shared" si="1"/>
-        <v>199.5</v>
+        <v>256.5</v>
       </c>
       <c r="E72">
         <f t="shared" si="2"/>
-        <v>300</v>
+        <v>375</v>
       </c>
       <c r="F72">
         <f t="shared" si="3"/>
-        <v>449.50000000000006</v>
+        <v>496</v>
       </c>
       <c r="G72">
         <f t="shared" si="4"/>
@@ -12774,19 +12971,19 @@
       <c r="A73" s="1"/>
       <c r="C73">
         <f t="shared" si="0"/>
-        <v>117</v>
+        <v>156</v>
       </c>
       <c r="D73">
         <f t="shared" si="1"/>
-        <v>199.5</v>
+        <v>256.5</v>
       </c>
       <c r="E73">
         <f t="shared" si="2"/>
-        <v>300</v>
+        <v>375</v>
       </c>
       <c r="F73">
         <f t="shared" si="3"/>
-        <v>449.50000000000006</v>
+        <v>496</v>
       </c>
       <c r="G73">
         <f t="shared" si="4"/>
@@ -12980,18 +13177,18 @@
         <v>73</v>
       </c>
       <c r="C8" s="9">
-        <v>0.09</v>
+        <v>0.12</v>
       </c>
       <c r="D8" s="8">
         <f t="shared" si="0"/>
-        <v>0.105</v>
+        <v>0.13500000000000001</v>
       </c>
       <c r="E8" s="9">
-        <v>0.12</v>
+        <v>0.15</v>
       </c>
       <c r="F8" s="8">
         <f t="shared" si="1"/>
-        <v>0.14500000000000002</v>
+        <v>0.16</v>
       </c>
       <c r="G8" s="9">
         <v>0.17</v>
@@ -13013,21 +13210,21 @@
         <v>76</v>
       </c>
       <c r="C9" s="9">
-        <v>0.72</v>
+        <v>0.78</v>
       </c>
       <c r="D9" s="8">
         <f t="shared" si="0"/>
-        <v>0.76</v>
+        <v>0.81</v>
       </c>
       <c r="E9" s="9">
-        <v>0.8</v>
+        <v>0.84</v>
       </c>
       <c r="F9" s="8">
         <f t="shared" si="1"/>
-        <v>0.84000000000000008</v>
+        <v>0.87</v>
       </c>
       <c r="G9" s="9">
-        <v>0.88</v>
+        <v>0.9</v>
       </c>
       <c r="H9" s="1" t="s">
         <v>77</v>
@@ -13079,19 +13276,19 @@
         <v>80</v>
       </c>
       <c r="C11" s="9">
-        <v>0.56000000000000005</v>
+        <v>0.57999999999999996</v>
       </c>
       <c r="D11" s="8">
-        <v>0.57999999999999996</v>
+        <v>0.59</v>
       </c>
       <c r="E11" s="9">
         <v>0.6</v>
       </c>
       <c r="F11" s="8">
+        <v>0.61</v>
+      </c>
+      <c r="G11" s="9">
         <v>0.62</v>
-      </c>
-      <c r="G11" s="9">
-        <v>0.64</v>
       </c>
       <c r="H11" s="1" t="s">
         <v>74</v>
@@ -13243,7 +13440,7 @@
     <row r="20" spans="1:13" ht="24" customHeight="1">
       <c r="A20" s="1"/>
       <c r="B20" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C20" s="1"/>
       <c r="D20" s="1"/>
@@ -13311,7 +13508,7 @@
     <row r="24" spans="1:13" ht="24" customHeight="1">
       <c r="A24" s="1"/>
       <c r="B24" s="1" t="s">
-        <v>89</v>
+        <v>103</v>
       </c>
       <c r="C24" s="1"/>
       <c r="D24" s="1"/>
@@ -13328,7 +13525,7 @@
     <row r="25" spans="1:13" ht="24" customHeight="1">
       <c r="A25" s="1"/>
       <c r="B25" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C25" s="1"/>
       <c r="D25" s="1"/>
@@ -13437,7 +13634,7 @@
     <row r="30" spans="1:13" ht="27" customHeight="1">
       <c r="A30" s="1"/>
       <c r="B30" s="20" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C30" s="22">
         <f t="shared" si="2"/>
@@ -13470,7 +13667,7 @@
     <row r="31" spans="1:13" ht="27" customHeight="1">
       <c r="A31" s="1"/>
       <c r="B31" s="20" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C31" s="26">
         <v>0.3</v>
@@ -13501,7 +13698,7 @@
     <row r="32" spans="1:13" ht="27" customHeight="1">
       <c r="A32" s="1"/>
       <c r="B32" s="20" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C32" s="26">
         <v>0.74</v>
@@ -13547,7 +13744,7 @@
     <row r="34" spans="1:13" ht="27" customHeight="1">
       <c r="A34" s="1"/>
       <c r="B34" s="20" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C34" s="20"/>
       <c r="D34" s="20"/>
@@ -13568,19 +13765,19 @@
     <row r="35" spans="1:13" ht="27" customHeight="1">
       <c r="A35" s="1"/>
       <c r="B35" s="20" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C35" s="20"/>
       <c r="D35" s="20"/>
       <c r="E35" s="25" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="F35" s="20"/>
       <c r="G35" s="20"/>
       <c r="H35" s="20"/>
       <c r="I35" s="20"/>
       <c r="J35" s="20" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="K35" s="1"/>
       <c r="L35" s="1"/>
@@ -13619,7 +13816,7 @@
     <row r="38" spans="1:13" ht="27" customHeight="1">
       <c r="A38" s="1"/>
       <c r="B38" s="20" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C38" s="20"/>
       <c r="D38" s="20"/>
@@ -13636,7 +13833,7 @@
     <row r="39" spans="1:13" ht="27" customHeight="1">
       <c r="A39" s="1"/>
       <c r="B39" s="20" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C39" s="20"/>
       <c r="D39" s="20"/>
@@ -13653,7 +13850,7 @@
     <row r="40" spans="1:13" ht="27" customHeight="1">
       <c r="A40" s="1"/>
       <c r="B40" s="20" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C40" s="20"/>
       <c r="D40" s="20"/>
@@ -13670,7 +13867,7 @@
     <row r="41" spans="1:13" ht="27" customHeight="1">
       <c r="A41" s="1"/>
       <c r="B41" s="20" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C41" s="20"/>
       <c r="D41" s="20"/>
@@ -13687,7 +13884,7 @@
     <row r="42" spans="1:13" ht="27" customHeight="1">
       <c r="A42" s="1"/>
       <c r="B42" s="20" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C42" s="20"/>
       <c r="D42" s="20"/>
@@ -14185,4 +14382,595 @@
   <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+  <dimension ref="A1:J30"/>
+  <sheetFormatPr defaultRowHeight="14"/>
+  <cols>
+    <col min="1" max="1" width="3" customWidth="1"/>
+    <col min="2" max="2" width="25" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="4" width="17" customWidth="1"/>
+    <col min="5" max="5" width="3" customWidth="1"/>
+    <col min="6" max="6" width="23" customWidth="1"/>
+    <col min="7" max="8" width="16" customWidth="1"/>
+    <col min="9" max="10" width="3" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" ht="25" customHeight="1">
+      <c r="A1" s="39"/>
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
+      <c r="G1" s="39"/>
+      <c r="H1" s="39"/>
+      <c r="I1" s="39"/>
+      <c r="J1" s="39"/>
+    </row>
+    <row r="2" spans="1:10" ht="25" customHeight="1">
+      <c r="A2" s="39"/>
+      <c r="B2" s="40" t="s">
+        <v>104</v>
+      </c>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="39"/>
+      <c r="H2" s="39"/>
+      <c r="I2" s="39"/>
+      <c r="J2" s="39"/>
+    </row>
+    <row r="3" spans="1:10" ht="25" customHeight="1">
+      <c r="A3" s="39"/>
+      <c r="B3" s="39"/>
+      <c r="C3" s="39"/>
+      <c r="D3" s="39"/>
+      <c r="E3" s="39"/>
+      <c r="F3" s="39"/>
+      <c r="G3" s="39"/>
+      <c r="H3" s="39"/>
+      <c r="I3" s="39"/>
+      <c r="J3" s="39"/>
+    </row>
+    <row r="4" spans="1:10" ht="28" customHeight="1">
+      <c r="A4" s="39"/>
+      <c r="B4" s="47" t="s">
+        <v>105</v>
+      </c>
+      <c r="C4" s="47" t="s">
+        <v>106</v>
+      </c>
+      <c r="D4" s="47" t="s">
+        <v>107</v>
+      </c>
+      <c r="E4" s="39"/>
+      <c r="F4" s="47" t="s">
+        <v>108</v>
+      </c>
+      <c r="G4" s="47" t="s">
+        <v>109</v>
+      </c>
+      <c r="H4" s="47" t="s">
+        <v>69</v>
+      </c>
+      <c r="I4" s="39"/>
+      <c r="J4" s="39"/>
+    </row>
+    <row r="5" spans="1:10" ht="25" customHeight="1">
+      <c r="A5" s="39"/>
+      <c r="B5" s="39" t="s">
+        <v>110</v>
+      </c>
+      <c r="C5" s="41" t="s">
+        <v>111</v>
+      </c>
+      <c r="D5" s="39" t="s">
+        <v>112</v>
+      </c>
+      <c r="E5" s="39"/>
+      <c r="F5" s="39" t="s">
+        <v>113</v>
+      </c>
+      <c r="G5" s="45">
+        <f>IF(AND(OR(C5="Rally2",C5="WRC17",C5="Rally1"),COUNT(C6:C9)=4,C6+C16&gt;=0,C6&lt;=0,C7+20&gt;=0,C7&lt;=0,C8+C17&gt;=0,C8&lt;=0,C9&gt;=0,C6=INT(C6),C7=INT(C7),C8=INT(C8)),G9*MIN(C9,G17)+G10*MAX(0,C9-G17)+G11*MAX(0,C9-G18),"检查输入")</f>
+        <v>3160</v>
+      </c>
+      <c r="H5" s="39" t="s">
+        <v>114</v>
+      </c>
+      <c r="I5" s="39"/>
+      <c r="J5" s="39"/>
+    </row>
+    <row r="6" spans="1:10" ht="25" customHeight="1">
+      <c r="A6" s="39"/>
+      <c r="B6" s="39" t="s">
+        <v>115</v>
+      </c>
+      <c r="C6" s="42">
+        <v>-12</v>
+      </c>
+      <c r="D6" s="39" t="str">
+        <f>"−"&amp;C16&amp;"～0 格"</f>
+        <v>−24～0 格</v>
+      </c>
+      <c r="E6" s="39"/>
+      <c r="F6" s="39" t="s">
+        <v>116</v>
+      </c>
+      <c r="G6" s="45">
+        <f>IF(AND(OR(C5="Rally2",C5="WRC17",C5="Rally1"),COUNT(C6:C9)=4,C6+C16&gt;=0,C6&lt;=0,C7+20&gt;=0,C7&lt;=0,C8+C17&gt;=0,C8&lt;=0,C9&gt;=0,C6=INT(C6),C7=INT(C7),C8=INT(C8)),G14*MIN(C9,G19)+G15*MAX(0,C9-G19),"检查输入")</f>
+        <v>1867.5450000000001</v>
+      </c>
+      <c r="H6" s="39" t="s">
+        <v>114</v>
+      </c>
+      <c r="I6" s="39"/>
+      <c r="J6" s="39"/>
+    </row>
+    <row r="7" spans="1:10" ht="25" customHeight="1">
+      <c r="A7" s="39"/>
+      <c r="B7" s="39" t="s">
+        <v>117</v>
+      </c>
+      <c r="C7" s="42">
+        <v>-10</v>
+      </c>
+      <c r="D7" s="39" t="s">
+        <v>118</v>
+      </c>
+      <c r="E7" s="39"/>
+      <c r="F7" s="39"/>
+      <c r="G7" s="39"/>
+      <c r="H7" s="39"/>
+      <c r="I7" s="39"/>
+      <c r="J7" s="39"/>
+    </row>
+    <row r="8" spans="1:10" ht="28" customHeight="1">
+      <c r="A8" s="39"/>
+      <c r="B8" s="39" t="s">
+        <v>119</v>
+      </c>
+      <c r="C8" s="42">
+        <v>-20</v>
+      </c>
+      <c r="D8" s="39" t="str">
+        <f>"−"&amp;C17&amp;"～0 格"</f>
+        <v>−40～0 格</v>
+      </c>
+      <c r="E8" s="39"/>
+      <c r="F8" s="47" t="s">
+        <v>120</v>
+      </c>
+      <c r="G8" s="47" t="s">
+        <v>106</v>
+      </c>
+      <c r="H8" s="47" t="s">
+        <v>69</v>
+      </c>
+      <c r="I8" s="39"/>
+      <c r="J8" s="39"/>
+    </row>
+    <row r="9" spans="1:10" ht="25" customHeight="1">
+      <c r="A9" s="39"/>
+      <c r="B9" s="39" t="s">
+        <v>121</v>
+      </c>
+      <c r="C9" s="43">
+        <v>1</v>
+      </c>
+      <c r="D9" s="39" t="s">
+        <v>74</v>
+      </c>
+      <c r="E9" s="39"/>
+      <c r="F9" s="39" t="s">
+        <v>122</v>
+      </c>
+      <c r="G9" s="44">
+        <f>INDEX(Parameters!$C$7:$G$7,1,C21)+(C18-INDEX(Parameters!$C$6:$G$6,1,C21))*(INDEX(Parameters!$C$7:$G$7,1,C21+1)-INDEX(Parameters!$C$7:$G$7,1,C21))/(INDEX(Parameters!$C$6:$G$6,1,C21+1)-INDEX(Parameters!$C$6:$G$6,1,C21))</f>
+        <v>2500</v>
+      </c>
+      <c r="H9" s="39" t="s">
+        <v>71</v>
+      </c>
+      <c r="I9" s="39"/>
+      <c r="J9" s="39"/>
+    </row>
+    <row r="10" spans="1:10" ht="25" customHeight="1">
+      <c r="A10" s="39"/>
+      <c r="B10" s="39"/>
+      <c r="C10" s="39"/>
+      <c r="D10" s="39"/>
+      <c r="E10" s="39"/>
+      <c r="F10" s="39" t="s">
+        <v>123</v>
+      </c>
+      <c r="G10" s="44">
+        <f>G9*(INDEX(Parameters!$C$9:$G$9,1,C21)+(C18-INDEX(Parameters!$C$6:$G$6,1,C21))*(INDEX(Parameters!$C$9:$G$9,1,C21+1)-INDEX(Parameters!$C$9:$G$9,1,C21))/(INDEX(Parameters!$C$6:$G$6,1,C21+1)-INDEX(Parameters!$C$6:$G$6,1,C21)))</f>
+        <v>2100</v>
+      </c>
+      <c r="H10" s="39" t="s">
+        <v>71</v>
+      </c>
+      <c r="I10" s="39"/>
+      <c r="J10" s="39"/>
+    </row>
+    <row r="11" spans="1:10" ht="25" customHeight="1">
+      <c r="A11" s="39"/>
+      <c r="B11" s="39"/>
+      <c r="C11" s="39"/>
+      <c r="D11" s="39"/>
+      <c r="E11" s="39"/>
+      <c r="F11" s="39" t="s">
+        <v>124</v>
+      </c>
+      <c r="G11" s="44">
+        <f>INDEX(Parameters!$C$10:$G$10,1,C22)+(C19-INDEX(Parameters!$C$6:$G$6,1,C22))*(INDEX(Parameters!$C$10:$G$10,1,C22+1)-INDEX(Parameters!$C$10:$G$10,1,C22))/(INDEX(Parameters!$C$6:$G$6,1,C22+1)-INDEX(Parameters!$C$6:$G$6,1,C22))</f>
+        <v>2500</v>
+      </c>
+      <c r="H11" s="39" t="s">
+        <v>71</v>
+      </c>
+      <c r="I11" s="39"/>
+      <c r="J11" s="39"/>
+    </row>
+    <row r="12" spans="1:10" ht="25" customHeight="1">
+      <c r="A12" s="39"/>
+      <c r="B12" s="39"/>
+      <c r="C12" s="39"/>
+      <c r="D12" s="39"/>
+      <c r="E12" s="39"/>
+      <c r="F12" s="39" t="s">
+        <v>125</v>
+      </c>
+      <c r="G12" s="44">
+        <f>G10+G11</f>
+        <v>4600</v>
+      </c>
+      <c r="H12" s="39" t="s">
+        <v>71</v>
+      </c>
+      <c r="I12" s="39"/>
+      <c r="J12" s="39"/>
+    </row>
+    <row r="13" spans="1:10" ht="25" customHeight="1">
+      <c r="A13" s="39"/>
+      <c r="B13" s="39"/>
+      <c r="C13" s="39"/>
+      <c r="D13" s="39"/>
+      <c r="E13" s="39"/>
+      <c r="F13" s="39"/>
+      <c r="G13" s="44"/>
+      <c r="H13" s="39"/>
+      <c r="I13" s="39"/>
+      <c r="J13" s="39"/>
+    </row>
+    <row r="14" spans="1:10" ht="28" customHeight="1">
+      <c r="A14" s="39"/>
+      <c r="B14" s="47" t="s">
+        <v>126</v>
+      </c>
+      <c r="C14" s="47" t="s">
+        <v>106</v>
+      </c>
+      <c r="D14" s="47" t="s">
+        <v>127</v>
+      </c>
+      <c r="E14" s="39"/>
+      <c r="F14" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="G14" s="44">
+        <f>INDEX(Parameters!$C$30:$G$30,1,C23)+(C20-INDEX(Parameters!$C$28:$G$28,1,C23))*(INDEX(Parameters!$C$30:$G$30,1,C23+1)-INDEX(Parameters!$C$30:$G$30,1,C23))/(INDEX(Parameters!$C$28:$G$28,1,C23+1)-INDEX(Parameters!$C$28:$G$28,1,C23))</f>
+        <v>2115</v>
+      </c>
+      <c r="H14" s="39" t="s">
+        <v>71</v>
+      </c>
+      <c r="I14" s="39"/>
+      <c r="J14" s="39"/>
+    </row>
+    <row r="15" spans="1:10" ht="25" customHeight="1">
+      <c r="A15" s="39"/>
+      <c r="B15" s="39"/>
+      <c r="C15" s="39"/>
+      <c r="D15" s="39"/>
+      <c r="E15" s="39"/>
+      <c r="F15" s="39" t="s">
+        <v>129</v>
+      </c>
+      <c r="G15" s="44">
+        <f>G14*(INDEX(Parameters!$C$32:$G$32,1,C23)+(C20-INDEX(Parameters!$C$28:$G$28,1,C23))*(INDEX(Parameters!$C$32:$G$32,1,C23+1)-INDEX(Parameters!$C$32:$G$32,1,C23))/(INDEX(Parameters!$C$28:$G$28,1,C23+1)-INDEX(Parameters!$C$28:$G$28,1,C23)))</f>
+        <v>1734.3</v>
+      </c>
+      <c r="H15" s="39" t="s">
+        <v>71</v>
+      </c>
+      <c r="I15" s="39"/>
+      <c r="J15" s="39"/>
+    </row>
+    <row r="16" spans="1:10" ht="25" customHeight="1">
+      <c r="A16" s="39"/>
+      <c r="B16" s="39" t="s">
+        <v>130</v>
+      </c>
+      <c r="C16" s="39">
+        <v>24</v>
+      </c>
+      <c r="D16" s="39" t="s">
+        <v>131</v>
+      </c>
+      <c r="E16" s="39"/>
+      <c r="F16" s="39"/>
+      <c r="G16" s="39"/>
+      <c r="H16" s="39"/>
+      <c r="I16" s="39"/>
+      <c r="J16" s="39"/>
+    </row>
+    <row r="17" spans="1:10" ht="25" customHeight="1">
+      <c r="A17" s="39"/>
+      <c r="B17" s="39" t="s">
+        <v>132</v>
+      </c>
+      <c r="C17" s="39">
+        <f>IF(C5="WRC17",60,40)</f>
+        <v>40</v>
+      </c>
+      <c r="D17" s="39" t="s">
+        <v>131</v>
+      </c>
+      <c r="E17" s="39"/>
+      <c r="F17" s="39" t="s">
+        <v>73</v>
+      </c>
+      <c r="G17" s="46">
+        <f>INDEX(Parameters!$C$8:$G$8,1,C21)+(C18-INDEX(Parameters!$C$6:$G$6,1,C21))*(INDEX(Parameters!$C$8:$G$8,1,C21+1)-INDEX(Parameters!$C$8:$G$8,1,C21))/(INDEX(Parameters!$C$6:$G$6,1,C21+1)-INDEX(Parameters!$C$6:$G$6,1,C21))</f>
+        <v>0.15</v>
+      </c>
+      <c r="H17" s="39" t="s">
+        <v>74</v>
+      </c>
+      <c r="I17" s="39"/>
+      <c r="J17" s="39"/>
+    </row>
+    <row r="18" spans="1:10" ht="25" customHeight="1">
+      <c r="A18" s="39"/>
+      <c r="B18" s="39" t="s">
+        <v>133</v>
+      </c>
+      <c r="C18" s="44">
+        <f>C6*20/C16</f>
+        <v>-10</v>
+      </c>
+      <c r="D18" s="39" t="s">
+        <v>134</v>
+      </c>
+      <c r="E18" s="39"/>
+      <c r="F18" s="39" t="s">
+        <v>80</v>
+      </c>
+      <c r="G18" s="46">
+        <f>INDEX(Parameters!$C$11:$G$11,1,C22)+(C19-INDEX(Parameters!$C$6:$G$6,1,C22))*(INDEX(Parameters!$C$11:$G$11,1,C22+1)-INDEX(Parameters!$C$11:$G$11,1,C22))/(INDEX(Parameters!$C$6:$G$6,1,C22+1)-INDEX(Parameters!$C$6:$G$6,1,C22))</f>
+        <v>0.6</v>
+      </c>
+      <c r="H18" s="39" t="s">
+        <v>74</v>
+      </c>
+      <c r="I18" s="39"/>
+      <c r="J18" s="39"/>
+    </row>
+    <row r="19" spans="1:10" ht="25" customHeight="1">
+      <c r="A19" s="39"/>
+      <c r="B19" s="39" t="s">
+        <v>135</v>
+      </c>
+      <c r="C19" s="44">
+        <f>C7</f>
+        <v>-10</v>
+      </c>
+      <c r="D19" s="39" t="s">
+        <v>136</v>
+      </c>
+      <c r="E19" s="39"/>
+      <c r="F19" s="39" t="s">
+        <v>92</v>
+      </c>
+      <c r="G19" s="46">
+        <f>INDEX(Parameters!$C$31:$G$31,1,C23)+(C20-INDEX(Parameters!$C$28:$G$28,1,C23))*(INDEX(Parameters!$C$31:$G$31,1,C23+1)-INDEX(Parameters!$C$31:$G$31,1,C23))/(INDEX(Parameters!$C$28:$G$28,1,C23+1)-INDEX(Parameters!$C$28:$G$28,1,C23))</f>
+        <v>0.35</v>
+      </c>
+      <c r="H19" s="39" t="s">
+        <v>74</v>
+      </c>
+      <c r="I19" s="39"/>
+      <c r="J19" s="39"/>
+    </row>
+    <row r="20" spans="1:10" ht="25" customHeight="1">
+      <c r="A20" s="39"/>
+      <c r="B20" s="39" t="s">
+        <v>137</v>
+      </c>
+      <c r="C20" s="44">
+        <f>C8*40/C17</f>
+        <v>-20</v>
+      </c>
+      <c r="D20" s="39" t="s">
+        <v>138</v>
+      </c>
+      <c r="E20" s="39"/>
+      <c r="F20" s="39"/>
+      <c r="G20" s="39"/>
+      <c r="H20" s="39"/>
+      <c r="I20" s="39"/>
+      <c r="J20" s="39"/>
+    </row>
+    <row r="21" spans="1:10" ht="25" customHeight="1">
+      <c r="A21" s="39"/>
+      <c r="B21" s="39" t="s">
+        <v>139</v>
+      </c>
+      <c r="C21" s="39">
+        <f>MIN(4,MATCH(C18,Parameters!$C$6:$G$6,1))</f>
+        <v>3</v>
+      </c>
+      <c r="D21" s="39"/>
+      <c r="E21" s="39"/>
+      <c r="F21" s="39"/>
+      <c r="G21" s="39"/>
+      <c r="H21" s="39"/>
+      <c r="I21" s="39"/>
+      <c r="J21" s="39"/>
+    </row>
+    <row r="22" spans="1:10" ht="25" customHeight="1">
+      <c r="A22" s="39"/>
+      <c r="B22" s="39" t="s">
+        <v>140</v>
+      </c>
+      <c r="C22" s="39">
+        <f>MIN(4,MATCH(C19,Parameters!$C$6:$G$6,1))</f>
+        <v>3</v>
+      </c>
+      <c r="D22" s="39"/>
+      <c r="E22" s="39"/>
+      <c r="F22" s="39"/>
+      <c r="G22" s="39"/>
+      <c r="H22" s="39"/>
+      <c r="I22" s="39"/>
+      <c r="J22" s="39"/>
+    </row>
+    <row r="23" spans="1:10" ht="25" customHeight="1">
+      <c r="A23" s="39"/>
+      <c r="B23" s="39" t="s">
+        <v>141</v>
+      </c>
+      <c r="C23" s="39">
+        <f>MIN(4,MATCH(C20,Parameters!$C$28:$G$28,1))</f>
+        <v>3</v>
+      </c>
+      <c r="D23" s="39"/>
+      <c r="E23" s="39"/>
+      <c r="F23" s="39"/>
+      <c r="G23" s="39"/>
+      <c r="H23" s="39"/>
+      <c r="I23" s="39"/>
+      <c r="J23" s="39"/>
+    </row>
+    <row r="24" spans="1:10" ht="25" customHeight="1">
+      <c r="A24" s="39"/>
+      <c r="B24" s="39"/>
+      <c r="C24" s="39"/>
+      <c r="D24" s="39"/>
+      <c r="E24" s="39"/>
+      <c r="F24" s="39"/>
+      <c r="G24" s="39"/>
+      <c r="H24" s="39"/>
+      <c r="I24" s="39"/>
+      <c r="J24" s="39"/>
+    </row>
+    <row r="25" spans="1:10" ht="25" customHeight="1">
+      <c r="A25" s="39"/>
+      <c r="B25" s="48" t="s">
+        <v>142</v>
+      </c>
+      <c r="C25" s="48"/>
+      <c r="D25" s="48"/>
+      <c r="E25" s="48"/>
+      <c r="F25" s="48"/>
+      <c r="G25" s="48"/>
+      <c r="H25" s="48"/>
+      <c r="I25" s="39"/>
+      <c r="J25" s="39"/>
+    </row>
+    <row r="26" spans="1:10" ht="25" customHeight="1">
+      <c r="A26" s="39"/>
+      <c r="B26" s="48" t="s">
+        <v>143</v>
+      </c>
+      <c r="C26" s="48"/>
+      <c r="D26" s="48"/>
+      <c r="E26" s="48"/>
+      <c r="F26" s="48"/>
+      <c r="G26" s="48"/>
+      <c r="H26" s="48"/>
+      <c r="I26" s="39"/>
+      <c r="J26" s="39"/>
+    </row>
+    <row r="27" spans="1:10" ht="25" customHeight="1">
+      <c r="A27" s="39"/>
+      <c r="B27" s="48" t="s">
+        <v>144</v>
+      </c>
+      <c r="C27" s="48"/>
+      <c r="D27" s="48"/>
+      <c r="E27" s="48"/>
+      <c r="F27" s="48"/>
+      <c r="G27" s="48"/>
+      <c r="H27" s="48"/>
+      <c r="I27" s="39"/>
+      <c r="J27" s="39"/>
+    </row>
+    <row r="28" spans="1:10" ht="25" customHeight="1">
+      <c r="A28" s="39"/>
+      <c r="B28" s="39"/>
+      <c r="C28" s="39"/>
+      <c r="D28" s="39"/>
+      <c r="E28" s="39"/>
+      <c r="F28" s="39"/>
+      <c r="G28" s="39"/>
+      <c r="H28" s="39"/>
+      <c r="I28" s="39"/>
+      <c r="J28" s="39"/>
+    </row>
+    <row r="29" spans="1:10" ht="25" customHeight="1">
+      <c r="A29" s="39"/>
+      <c r="B29" s="39"/>
+      <c r="C29" s="39"/>
+      <c r="D29" s="39"/>
+      <c r="E29" s="39"/>
+      <c r="F29" s="39"/>
+      <c r="G29" s="39"/>
+      <c r="H29" s="39"/>
+      <c r="I29" s="39"/>
+      <c r="J29" s="39"/>
+    </row>
+    <row r="30" spans="1:10" ht="25" customHeight="1">
+      <c r="A30" s="39"/>
+      <c r="B30" s="39"/>
+      <c r="C30" s="39"/>
+      <c r="D30" s="39"/>
+      <c r="E30" s="39"/>
+      <c r="F30" s="39"/>
+      <c r="G30" s="39"/>
+      <c r="H30" s="39"/>
+      <c r="I30" s="39"/>
+      <c r="J30" s="39"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="7" type="noConversion"/>
+  <dataValidations count="5">
+    <dataValidation type="list" sqref="C5" xr:uid="{00000000-0002-0000-0500-000000000000}">
+      <formula1>"Rally2,WRC17,Rally1"</formula1>
+    </dataValidation>
+    <dataValidation type="whole" sqref="C6" xr:uid="{00000000-0002-0000-0500-000001000000}">
+      <formula1>-C16</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation type="whole" sqref="C7" xr:uid="{00000000-0002-0000-0500-000002000000}">
+      <formula1>-20</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation type="whole" sqref="C8" xr:uid="{00000000-0002-0000-0500-000003000000}">
+      <formula1>-C17</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" operator="greaterThanOrEqual" sqref="C9" xr:uid="{00000000-0002-0000-0500-000004000000}">
+      <formula1>0</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
damping and naming change
</commit_message>
<xml_diff>
--- a/docs/damping_curve.xlsx
+++ b/docs/damping_curve.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5DCEB5D-1A26-4980-AE5D-B24DCA0DE274}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Calculator" sheetId="6" r:id="rId1"/>
@@ -483,10 +483,22 @@
     <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
@@ -495,20 +507,8 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="2" fontId="11" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -6126,20 +6126,20 @@
     </row>
     <row r="2" spans="1:15" ht="23" customHeight="1">
       <c r="A2" s="1"/>
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
-      <c r="E2" s="20"/>
-      <c r="F2" s="20"/>
-      <c r="G2" s="20"/>
-      <c r="H2" s="20"/>
-      <c r="I2" s="20"/>
-      <c r="J2" s="20"/>
-      <c r="K2" s="20"/>
-      <c r="L2" s="20"/>
-      <c r="M2" s="20"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
+      <c r="H2" s="22"/>
+      <c r="I2" s="22"/>
+      <c r="J2" s="22"/>
+      <c r="K2" s="22"/>
+      <c r="L2" s="22"/>
+      <c r="M2" s="22"/>
       <c r="N2" s="1"/>
       <c r="O2" s="1"/>
     </row>
@@ -6169,17 +6169,17 @@
         <v>2</v>
       </c>
       <c r="D4" s="1"/>
-      <c r="E4" s="21" t="s">
+      <c r="E4" s="25" t="s">
         <v>45</v>
       </c>
-      <c r="F4" s="21"/>
-      <c r="G4" s="21"/>
-      <c r="H4" s="21"/>
-      <c r="I4" s="21"/>
-      <c r="J4" s="21"/>
-      <c r="K4" s="21"/>
-      <c r="L4" s="21"/>
-      <c r="M4" s="21"/>
+      <c r="F4" s="25"/>
+      <c r="G4" s="25"/>
+      <c r="H4" s="25"/>
+      <c r="I4" s="25"/>
+      <c r="J4" s="25"/>
+      <c r="K4" s="25"/>
+      <c r="L4" s="25"/>
+      <c r="M4" s="25"/>
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
     </row>
@@ -6210,13 +6210,13 @@
       </c>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
-      <c r="F6" s="23" t="s">
+      <c r="F6" s="20" t="s">
         <v>48</v>
       </c>
-      <c r="G6" s="23"/>
-      <c r="H6" s="23"/>
-      <c r="I6" s="23"/>
-      <c r="J6" s="23"/>
+      <c r="G6" s="20"/>
+      <c r="H6" s="20"/>
+      <c r="I6" s="20"/>
+      <c r="J6" s="20"/>
       <c r="K6" s="1"/>
       <c r="L6" s="1"/>
       <c r="M6" s="1"/>
@@ -6254,16 +6254,16 @@
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
-      <c r="F8" s="20" t="s">
+      <c r="F8" s="22" t="s">
         <v>49</v>
       </c>
-      <c r="G8" s="20"/>
-      <c r="H8" s="20"/>
-      <c r="I8" s="24">
+      <c r="G8" s="22"/>
+      <c r="H8" s="22"/>
+      <c r="I8" s="27">
         <f>IF(C18="OK",Samples!F165*MIN(C10,Samples!G165)+Samples!I165*MAX(0,C10-Samples!G165)+Samples!J165*MAX(0,C10-Samples!K165),"检查输入")</f>
         <v>2228</v>
       </c>
-      <c r="J8" s="24"/>
+      <c r="J8" s="27"/>
       <c r="K8" s="1"/>
       <c r="L8" s="1"/>
       <c r="M8" s="1"/>
@@ -6301,16 +6301,16 @@
       </c>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
-      <c r="F10" s="20" t="s">
+      <c r="F10" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="G10" s="20"/>
-      <c r="H10" s="20"/>
-      <c r="I10" s="24">
+      <c r="G10" s="22"/>
+      <c r="H10" s="22"/>
+      <c r="I10" s="27">
         <f>IF(C18="OK",Samples!M165*MIN(C10,Samples!N165)+Samples!P165*MAX(0,C10-Samples!N165),"检查输入")</f>
         <v>1392</v>
       </c>
-      <c r="J10" s="24"/>
+      <c r="J10" s="27"/>
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
       <c r="M10" s="1"/>
@@ -6362,13 +6362,13 @@
       </c>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
-      <c r="F13" s="23" t="s">
+      <c r="F13" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="G13" s="23"/>
-      <c r="H13" s="23"/>
-      <c r="I13" s="23"/>
-      <c r="J13" s="23"/>
+      <c r="G13" s="20"/>
+      <c r="H13" s="20"/>
+      <c r="I13" s="20"/>
+      <c r="J13" s="20"/>
       <c r="K13" s="1"/>
       <c r="L13" s="1"/>
       <c r="M13" s="1"/>
@@ -6386,11 +6386,11 @@
       </c>
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
-      <c r="F14" s="20" t="s">
+      <c r="F14" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="G14" s="20"/>
-      <c r="H14" s="20"/>
+      <c r="G14" s="22"/>
+      <c r="H14" s="22"/>
       <c r="I14" s="18">
         <f>Samples!F165</f>
         <v>2500</v>
@@ -6415,11 +6415,11 @@
       </c>
       <c r="D15" s="1"/>
       <c r="E15" s="1"/>
-      <c r="F15" s="20" t="s">
+      <c r="F15" s="22" t="s">
         <v>57</v>
       </c>
-      <c r="G15" s="20"/>
-      <c r="H15" s="20"/>
+      <c r="G15" s="22"/>
+      <c r="H15" s="22"/>
       <c r="I15" s="18">
         <f>Samples!I165</f>
         <v>2100</v>
@@ -6439,11 +6439,11 @@
       <c r="C16" s="1"/>
       <c r="D16" s="1"/>
       <c r="E16" s="1"/>
-      <c r="F16" s="20" t="s">
+      <c r="F16" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="G16" s="20"/>
-      <c r="H16" s="20"/>
+      <c r="G16" s="22"/>
+      <c r="H16" s="22"/>
       <c r="I16" s="18">
         <f>Samples!J165</f>
         <v>2500</v>
@@ -6463,11 +6463,11 @@
       <c r="C17" s="1"/>
       <c r="D17" s="1"/>
       <c r="E17" s="1"/>
-      <c r="F17" s="20" t="s">
+      <c r="F17" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="G17" s="20"/>
-      <c r="H17" s="20"/>
+      <c r="G17" s="22"/>
+      <c r="H17" s="22"/>
       <c r="I17" s="18">
         <f>Samples!L165</f>
         <v>4600</v>
@@ -6509,11 +6509,11 @@
       <c r="C19" s="1"/>
       <c r="D19" s="1"/>
       <c r="E19" s="1"/>
-      <c r="F19" s="20" t="s">
+      <c r="F19" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="G19" s="20"/>
-      <c r="H19" s="20"/>
+      <c r="G19" s="22"/>
+      <c r="H19" s="22"/>
       <c r="I19" s="18">
         <f>Samples!M165</f>
         <v>2000</v>
@@ -6533,11 +6533,11 @@
       <c r="C20" s="1"/>
       <c r="D20" s="1"/>
       <c r="E20" s="1"/>
-      <c r="F20" s="20" t="s">
+      <c r="F20" s="22" t="s">
         <v>60</v>
       </c>
-      <c r="G20" s="20"/>
-      <c r="H20" s="20"/>
+      <c r="G20" s="22"/>
+      <c r="H20" s="22"/>
       <c r="I20" s="18">
         <f>Samples!P165</f>
         <v>1600</v>
@@ -6574,11 +6574,11 @@
       <c r="C22" s="1"/>
       <c r="D22" s="1"/>
       <c r="E22" s="1"/>
-      <c r="F22" s="20" t="s">
+      <c r="F22" s="22" t="s">
         <v>82</v>
       </c>
-      <c r="G22" s="20"/>
-      <c r="H22" s="20"/>
+      <c r="G22" s="22"/>
+      <c r="H22" s="22"/>
       <c r="I22" s="5">
         <f>Samples!G165</f>
         <v>0.12</v>
@@ -6598,11 +6598,11 @@
       <c r="C23" s="1"/>
       <c r="D23" s="1"/>
       <c r="E23" s="1"/>
-      <c r="F23" s="20" t="s">
+      <c r="F23" s="22" t="s">
         <v>83</v>
       </c>
-      <c r="G23" s="20"/>
-      <c r="H23" s="20"/>
+      <c r="G23" s="22"/>
+      <c r="H23" s="22"/>
       <c r="I23" s="5">
         <f>Samples!K165</f>
         <v>0.6</v>
@@ -6622,11 +6622,11 @@
       <c r="C24" s="1"/>
       <c r="D24" s="1"/>
       <c r="E24" s="1"/>
-      <c r="F24" s="20" t="s">
+      <c r="F24" s="22" t="s">
         <v>29</v>
       </c>
-      <c r="G24" s="20"/>
-      <c r="H24" s="20"/>
+      <c r="G24" s="22"/>
+      <c r="H24" s="22"/>
       <c r="I24" s="5">
         <f>Samples!N165</f>
         <v>0.28000000000000003</v>
@@ -6676,20 +6676,20 @@
     </row>
     <row r="27" spans="1:15" ht="23" customHeight="1">
       <c r="A27" s="1"/>
-      <c r="B27" s="22" t="s">
+      <c r="B27" s="26" t="s">
         <v>61</v>
       </c>
-      <c r="C27" s="22"/>
-      <c r="D27" s="22"/>
-      <c r="E27" s="22"/>
-      <c r="F27" s="22"/>
-      <c r="G27" s="22"/>
-      <c r="H27" s="22"/>
-      <c r="I27" s="22"/>
-      <c r="J27" s="22"/>
-      <c r="K27" s="22"/>
-      <c r="L27" s="22"/>
-      <c r="M27" s="22"/>
+      <c r="C27" s="26"/>
+      <c r="D27" s="26"/>
+      <c r="E27" s="26"/>
+      <c r="F27" s="26"/>
+      <c r="G27" s="26"/>
+      <c r="H27" s="26"/>
+      <c r="I27" s="26"/>
+      <c r="J27" s="26"/>
+      <c r="K27" s="26"/>
+      <c r="L27" s="26"/>
+      <c r="M27" s="26"/>
       <c r="N27" s="1"/>
       <c r="O27" s="1"/>
     </row>
@@ -6950,17 +6950,6 @@
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="B27:M27"/>
-    <mergeCell ref="F19:H19"/>
-    <mergeCell ref="F20:H20"/>
-    <mergeCell ref="F22:H22"/>
-    <mergeCell ref="F23:H23"/>
-    <mergeCell ref="F24:H24"/>
-    <mergeCell ref="F13:J13"/>
-    <mergeCell ref="F14:H14"/>
-    <mergeCell ref="F15:H15"/>
-    <mergeCell ref="F16:H16"/>
-    <mergeCell ref="F17:H17"/>
     <mergeCell ref="B2:M2"/>
     <mergeCell ref="E4:M4"/>
     <mergeCell ref="F6:J6"/>
@@ -6968,6 +6957,17 @@
     <mergeCell ref="F10:H10"/>
     <mergeCell ref="I8:J8"/>
     <mergeCell ref="I10:J10"/>
+    <mergeCell ref="F13:J13"/>
+    <mergeCell ref="F14:H14"/>
+    <mergeCell ref="F15:H15"/>
+    <mergeCell ref="F16:H16"/>
+    <mergeCell ref="F17:H17"/>
+    <mergeCell ref="B27:M27"/>
+    <mergeCell ref="F19:H19"/>
+    <mergeCell ref="F20:H20"/>
+    <mergeCell ref="F22:H22"/>
+    <mergeCell ref="F23:H23"/>
+    <mergeCell ref="F24:H24"/>
   </mergeCells>
   <phoneticPr fontId="13" type="noConversion"/>
   <dataValidations count="6">
@@ -7028,20 +7028,20 @@
     </row>
     <row r="2" spans="1:15" ht="23" customHeight="1">
       <c r="A2" s="1"/>
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
-      <c r="E2" s="20"/>
-      <c r="F2" s="20"/>
-      <c r="G2" s="20"/>
-      <c r="H2" s="20"/>
-      <c r="I2" s="20"/>
-      <c r="J2" s="20"/>
-      <c r="K2" s="20"/>
-      <c r="L2" s="20"/>
-      <c r="M2" s="20"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
+      <c r="H2" s="22"/>
+      <c r="I2" s="22"/>
+      <c r="J2" s="22"/>
+      <c r="K2" s="22"/>
+      <c r="L2" s="22"/>
+      <c r="M2" s="22"/>
       <c r="N2" s="1"/>
       <c r="O2" s="1"/>
     </row>
@@ -7071,17 +7071,17 @@
         <v>2</v>
       </c>
       <c r="D4" s="1"/>
-      <c r="E4" s="21" t="s">
+      <c r="E4" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="F4" s="21"/>
-      <c r="G4" s="21"/>
-      <c r="H4" s="21"/>
-      <c r="I4" s="21"/>
-      <c r="J4" s="21"/>
-      <c r="K4" s="21"/>
-      <c r="L4" s="21"/>
-      <c r="M4" s="21"/>
+      <c r="F4" s="25"/>
+      <c r="G4" s="25"/>
+      <c r="H4" s="25"/>
+      <c r="I4" s="25"/>
+      <c r="J4" s="25"/>
+      <c r="K4" s="25"/>
+      <c r="L4" s="25"/>
+      <c r="M4" s="25"/>
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
     </row>
@@ -7111,17 +7111,17 @@
         <v>-10</v>
       </c>
       <c r="D6" s="1"/>
-      <c r="E6" s="20" t="s">
+      <c r="E6" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="F6" s="20"/>
-      <c r="G6" s="20"/>
-      <c r="H6" s="20"/>
-      <c r="I6" s="20"/>
-      <c r="J6" s="20"/>
-      <c r="K6" s="20"/>
-      <c r="L6" s="20"/>
-      <c r="M6" s="20"/>
+      <c r="F6" s="22"/>
+      <c r="G6" s="22"/>
+      <c r="H6" s="22"/>
+      <c r="I6" s="22"/>
+      <c r="J6" s="22"/>
+      <c r="K6" s="22"/>
+      <c r="L6" s="22"/>
+      <c r="M6" s="22"/>
       <c r="N6" s="1"/>
       <c r="O6" s="1"/>
     </row>
@@ -7705,20 +7705,20 @@
     </row>
     <row r="41" spans="1:15" ht="23" customHeight="1">
       <c r="A41" s="1"/>
-      <c r="B41" s="22" t="s">
+      <c r="B41" s="26" t="s">
         <v>6</v>
       </c>
-      <c r="C41" s="22"/>
-      <c r="D41" s="22"/>
-      <c r="E41" s="22"/>
-      <c r="F41" s="22"/>
-      <c r="G41" s="22"/>
-      <c r="H41" s="22"/>
-      <c r="I41" s="22"/>
-      <c r="J41" s="22"/>
-      <c r="K41" s="22"/>
-      <c r="L41" s="22"/>
-      <c r="M41" s="22"/>
+      <c r="C41" s="26"/>
+      <c r="D41" s="26"/>
+      <c r="E41" s="26"/>
+      <c r="F41" s="26"/>
+      <c r="G41" s="26"/>
+      <c r="H41" s="26"/>
+      <c r="I41" s="26"/>
+      <c r="J41" s="26"/>
+      <c r="K41" s="26"/>
+      <c r="L41" s="26"/>
+      <c r="M41" s="26"/>
       <c r="N41" s="1"/>
       <c r="O41" s="1"/>
     </row>
@@ -7792,20 +7792,20 @@
     </row>
     <row r="2" spans="1:15" ht="23" customHeight="1">
       <c r="A2" s="1"/>
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="24" t="s">
         <v>86</v>
       </c>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
-      <c r="E2" s="20"/>
-      <c r="F2" s="20"/>
-      <c r="G2" s="20"/>
-      <c r="H2" s="20"/>
-      <c r="I2" s="20"/>
-      <c r="J2" s="20"/>
-      <c r="K2" s="20"/>
-      <c r="L2" s="20"/>
-      <c r="M2" s="20"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
+      <c r="H2" s="22"/>
+      <c r="I2" s="22"/>
+      <c r="J2" s="22"/>
+      <c r="K2" s="22"/>
+      <c r="L2" s="22"/>
+      <c r="M2" s="22"/>
       <c r="N2" s="1"/>
       <c r="O2" s="1"/>
     </row>
@@ -7835,17 +7835,17 @@
         <v>81</v>
       </c>
       <c r="D4" s="1"/>
-      <c r="E4" s="21" t="s">
+      <c r="E4" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="F4" s="21"/>
-      <c r="G4" s="21"/>
-      <c r="H4" s="21"/>
-      <c r="I4" s="21"/>
-      <c r="J4" s="21"/>
-      <c r="K4" s="21"/>
-      <c r="L4" s="21"/>
-      <c r="M4" s="21"/>
+      <c r="F4" s="25"/>
+      <c r="G4" s="25"/>
+      <c r="H4" s="25"/>
+      <c r="I4" s="25"/>
+      <c r="J4" s="25"/>
+      <c r="K4" s="25"/>
+      <c r="L4" s="25"/>
+      <c r="M4" s="25"/>
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
     </row>
@@ -7875,17 +7875,17 @@
         <v>-12</v>
       </c>
       <c r="D6" s="1"/>
-      <c r="E6" s="20" t="s">
+      <c r="E6" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="F6" s="20"/>
-      <c r="G6" s="20"/>
-      <c r="H6" s="20"/>
-      <c r="I6" s="20"/>
-      <c r="J6" s="20"/>
-      <c r="K6" s="20"/>
-      <c r="L6" s="20"/>
-      <c r="M6" s="20"/>
+      <c r="F6" s="22"/>
+      <c r="G6" s="22"/>
+      <c r="H6" s="22"/>
+      <c r="I6" s="22"/>
+      <c r="J6" s="22"/>
+      <c r="K6" s="22"/>
+      <c r="L6" s="22"/>
+      <c r="M6" s="22"/>
       <c r="N6" s="1"/>
       <c r="O6" s="1"/>
     </row>
@@ -8469,20 +8469,20 @@
     </row>
     <row r="41" spans="1:15" ht="23" customHeight="1">
       <c r="A41" s="1"/>
-      <c r="B41" s="22" t="s">
+      <c r="B41" s="26" t="s">
         <v>6</v>
       </c>
-      <c r="C41" s="22"/>
-      <c r="D41" s="22"/>
-      <c r="E41" s="22"/>
-      <c r="F41" s="22"/>
-      <c r="G41" s="22"/>
-      <c r="H41" s="22"/>
-      <c r="I41" s="22"/>
-      <c r="J41" s="22"/>
-      <c r="K41" s="22"/>
-      <c r="L41" s="22"/>
-      <c r="M41" s="22"/>
+      <c r="C41" s="26"/>
+      <c r="D41" s="26"/>
+      <c r="E41" s="26"/>
+      <c r="F41" s="26"/>
+      <c r="G41" s="26"/>
+      <c r="H41" s="26"/>
+      <c r="I41" s="26"/>
+      <c r="J41" s="26"/>
+      <c r="K41" s="26"/>
+      <c r="L41" s="26"/>
+      <c r="M41" s="26"/>
       <c r="N41" s="1"/>
       <c r="O41" s="1"/>
     </row>
@@ -8556,20 +8556,20 @@
     </row>
     <row r="2" spans="1:15" ht="23" customHeight="1">
       <c r="A2" s="1"/>
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="24" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
-      <c r="E2" s="20"/>
-      <c r="F2" s="20"/>
-      <c r="G2" s="20"/>
-      <c r="H2" s="20"/>
-      <c r="I2" s="20"/>
-      <c r="J2" s="20"/>
-      <c r="K2" s="20"/>
-      <c r="L2" s="20"/>
-      <c r="M2" s="20"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
+      <c r="H2" s="22"/>
+      <c r="I2" s="22"/>
+      <c r="J2" s="22"/>
+      <c r="K2" s="22"/>
+      <c r="L2" s="22"/>
+      <c r="M2" s="22"/>
       <c r="N2" s="1"/>
       <c r="O2" s="1"/>
     </row>
@@ -8599,17 +8599,17 @@
         <v>2</v>
       </c>
       <c r="D4" s="1"/>
-      <c r="E4" s="21" t="s">
+      <c r="E4" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="F4" s="21"/>
-      <c r="G4" s="21"/>
-      <c r="H4" s="21"/>
-      <c r="I4" s="21"/>
-      <c r="J4" s="21"/>
-      <c r="K4" s="21"/>
-      <c r="L4" s="21"/>
-      <c r="M4" s="21"/>
+      <c r="F4" s="25"/>
+      <c r="G4" s="25"/>
+      <c r="H4" s="25"/>
+      <c r="I4" s="25"/>
+      <c r="J4" s="25"/>
+      <c r="K4" s="25"/>
+      <c r="L4" s="25"/>
+      <c r="M4" s="25"/>
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
     </row>
@@ -8632,20 +8632,20 @@
     </row>
     <row r="6" spans="1:15" ht="23" customHeight="1">
       <c r="A6" s="1"/>
-      <c r="B6" s="20" t="s">
+      <c r="B6" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="20"/>
-      <c r="D6" s="20"/>
-      <c r="E6" s="20"/>
-      <c r="F6" s="20"/>
-      <c r="G6" s="20"/>
-      <c r="H6" s="20"/>
-      <c r="I6" s="20"/>
-      <c r="J6" s="20"/>
-      <c r="K6" s="20"/>
-      <c r="L6" s="20"/>
-      <c r="M6" s="20"/>
+      <c r="C6" s="22"/>
+      <c r="D6" s="22"/>
+      <c r="E6" s="22"/>
+      <c r="F6" s="22"/>
+      <c r="G6" s="22"/>
+      <c r="H6" s="22"/>
+      <c r="I6" s="22"/>
+      <c r="J6" s="22"/>
+      <c r="K6" s="22"/>
+      <c r="L6" s="22"/>
+      <c r="M6" s="22"/>
       <c r="N6" s="1"/>
       <c r="O6" s="1"/>
     </row>
@@ -9229,20 +9229,20 @@
     </row>
     <row r="41" spans="1:15" ht="23" customHeight="1">
       <c r="A41" s="1"/>
-      <c r="B41" s="22" t="s">
+      <c r="B41" s="26" t="s">
         <v>6</v>
       </c>
-      <c r="C41" s="22"/>
-      <c r="D41" s="22"/>
-      <c r="E41" s="22"/>
-      <c r="F41" s="22"/>
-      <c r="G41" s="22"/>
-      <c r="H41" s="22"/>
-      <c r="I41" s="22"/>
-      <c r="J41" s="22"/>
-      <c r="K41" s="22"/>
-      <c r="L41" s="22"/>
-      <c r="M41" s="22"/>
+      <c r="C41" s="26"/>
+      <c r="D41" s="26"/>
+      <c r="E41" s="26"/>
+      <c r="F41" s="26"/>
+      <c r="G41" s="26"/>
+      <c r="H41" s="26"/>
+      <c r="I41" s="26"/>
+      <c r="J41" s="26"/>
+      <c r="K41" s="26"/>
+      <c r="L41" s="26"/>
+      <c r="M41" s="26"/>
       <c r="N41" s="1"/>
       <c r="O41" s="1"/>
     </row>
@@ -9312,20 +9312,20 @@
     </row>
     <row r="2" spans="1:15" ht="23" customHeight="1">
       <c r="A2" s="1"/>
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="24" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
-      <c r="E2" s="20"/>
-      <c r="F2" s="20"/>
-      <c r="G2" s="20"/>
-      <c r="H2" s="20"/>
-      <c r="I2" s="20"/>
-      <c r="J2" s="20"/>
-      <c r="K2" s="20"/>
-      <c r="L2" s="20"/>
-      <c r="M2" s="20"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
+      <c r="H2" s="22"/>
+      <c r="I2" s="22"/>
+      <c r="J2" s="22"/>
+      <c r="K2" s="22"/>
+      <c r="L2" s="22"/>
+      <c r="M2" s="22"/>
       <c r="N2" s="1"/>
       <c r="O2" s="1"/>
     </row>
@@ -9355,17 +9355,17 @@
         <v>2</v>
       </c>
       <c r="D4" s="1"/>
-      <c r="E4" s="21" t="s">
+      <c r="E4" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="F4" s="21"/>
-      <c r="G4" s="21"/>
-      <c r="H4" s="21"/>
-      <c r="I4" s="21"/>
-      <c r="J4" s="21"/>
-      <c r="K4" s="21"/>
-      <c r="L4" s="21"/>
-      <c r="M4" s="21"/>
+      <c r="F4" s="25"/>
+      <c r="G4" s="25"/>
+      <c r="H4" s="25"/>
+      <c r="I4" s="25"/>
+      <c r="J4" s="25"/>
+      <c r="K4" s="25"/>
+      <c r="L4" s="25"/>
+      <c r="M4" s="25"/>
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
     </row>
@@ -9388,20 +9388,20 @@
     </row>
     <row r="6" spans="1:15" ht="23" customHeight="1">
       <c r="A6" s="1"/>
-      <c r="B6" s="20" t="s">
+      <c r="B6" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="20"/>
-      <c r="D6" s="20"/>
-      <c r="E6" s="20"/>
-      <c r="F6" s="20"/>
-      <c r="G6" s="20"/>
-      <c r="H6" s="20"/>
-      <c r="I6" s="20"/>
-      <c r="J6" s="20"/>
-      <c r="K6" s="20"/>
-      <c r="L6" s="20"/>
-      <c r="M6" s="20"/>
+      <c r="C6" s="22"/>
+      <c r="D6" s="22"/>
+      <c r="E6" s="22"/>
+      <c r="F6" s="22"/>
+      <c r="G6" s="22"/>
+      <c r="H6" s="22"/>
+      <c r="I6" s="22"/>
+      <c r="J6" s="22"/>
+      <c r="K6" s="22"/>
+      <c r="L6" s="22"/>
+      <c r="M6" s="22"/>
       <c r="N6" s="1"/>
       <c r="O6" s="1"/>
     </row>
@@ -9985,20 +9985,20 @@
     </row>
     <row r="41" spans="1:15" ht="23" customHeight="1">
       <c r="A41" s="1"/>
-      <c r="B41" s="22" t="s">
+      <c r="B41" s="26" t="s">
         <v>6</v>
       </c>
-      <c r="C41" s="22"/>
-      <c r="D41" s="22"/>
-      <c r="E41" s="22"/>
-      <c r="F41" s="22"/>
-      <c r="G41" s="22"/>
-      <c r="H41" s="22"/>
-      <c r="I41" s="22"/>
-      <c r="J41" s="22"/>
-      <c r="K41" s="22"/>
-      <c r="L41" s="22"/>
-      <c r="M41" s="22"/>
+      <c r="C41" s="26"/>
+      <c r="D41" s="26"/>
+      <c r="E41" s="26"/>
+      <c r="F41" s="26"/>
+      <c r="G41" s="26"/>
+      <c r="H41" s="26"/>
+      <c r="I41" s="26"/>
+      <c r="J41" s="26"/>
+      <c r="K41" s="26"/>
+      <c r="L41" s="26"/>
+      <c r="M41" s="26"/>
       <c r="N41" s="1"/>
       <c r="O41" s="1"/>
     </row>
@@ -10072,40 +10072,40 @@
     </row>
     <row r="2" spans="1:15" ht="23" customHeight="1">
       <c r="A2" s="1"/>
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
-      <c r="E2" s="20"/>
-      <c r="F2" s="20"/>
-      <c r="G2" s="20"/>
-      <c r="H2" s="20"/>
-      <c r="I2" s="20"/>
-      <c r="J2" s="20"/>
-      <c r="K2" s="20"/>
-      <c r="L2" s="20"/>
-      <c r="M2" s="20"/>
-      <c r="N2" s="20"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
+      <c r="H2" s="22"/>
+      <c r="I2" s="22"/>
+      <c r="J2" s="22"/>
+      <c r="K2" s="22"/>
+      <c r="L2" s="22"/>
+      <c r="M2" s="22"/>
+      <c r="N2" s="22"/>
       <c r="O2" s="1"/>
     </row>
     <row r="3" spans="1:15" ht="23" customHeight="1">
       <c r="A3" s="1"/>
-      <c r="B3" s="21" t="s">
+      <c r="B3" s="25" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
-      <c r="F3" s="20"/>
-      <c r="G3" s="20"/>
-      <c r="H3" s="20"/>
-      <c r="I3" s="20"/>
-      <c r="J3" s="20"/>
-      <c r="K3" s="20"/>
-      <c r="L3" s="20"/>
-      <c r="M3" s="20"/>
-      <c r="N3" s="20"/>
+      <c r="C3" s="22"/>
+      <c r="D3" s="22"/>
+      <c r="E3" s="22"/>
+      <c r="F3" s="22"/>
+      <c r="G3" s="22"/>
+      <c r="H3" s="22"/>
+      <c r="I3" s="22"/>
+      <c r="J3" s="22"/>
+      <c r="K3" s="22"/>
+      <c r="L3" s="22"/>
+      <c r="M3" s="22"/>
+      <c r="N3" s="22"/>
       <c r="O3" s="1"/>
     </row>
     <row r="4" spans="1:15" ht="23" customHeight="1">
@@ -10129,21 +10129,21 @@
       <c r="A5" s="1"/>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
-      <c r="D5" s="23" t="s">
+      <c r="D5" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="E5" s="23"/>
-      <c r="F5" s="23"/>
-      <c r="G5" s="23"/>
-      <c r="H5" s="23"/>
+      <c r="E5" s="20"/>
+      <c r="F5" s="20"/>
+      <c r="G5" s="20"/>
+      <c r="H5" s="20"/>
       <c r="I5" s="1"/>
-      <c r="J5" s="23" t="s">
+      <c r="J5" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="K5" s="23"/>
-      <c r="L5" s="23"/>
-      <c r="M5" s="23"/>
-      <c r="N5" s="23"/>
+      <c r="K5" s="20"/>
+      <c r="L5" s="20"/>
+      <c r="M5" s="20"/>
+      <c r="N5" s="20"/>
       <c r="O5" s="1"/>
     </row>
     <row r="6" spans="1:15" ht="23" customHeight="1">
@@ -10775,73 +10775,73 @@
     </row>
     <row r="22" spans="1:15" ht="23" customHeight="1">
       <c r="A22" s="1"/>
-      <c r="B22" s="23" t="s">
+      <c r="B22" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="C22" s="23"/>
-      <c r="D22" s="23"/>
-      <c r="E22" s="23"/>
-      <c r="F22" s="23"/>
-      <c r="G22" s="23"/>
-      <c r="H22" s="23"/>
-      <c r="I22" s="23"/>
-      <c r="J22" s="23"/>
-      <c r="K22" s="23"/>
-      <c r="L22" s="23"/>
-      <c r="M22" s="23"/>
-      <c r="N22" s="23"/>
+      <c r="C22" s="20"/>
+      <c r="D22" s="20"/>
+      <c r="E22" s="20"/>
+      <c r="F22" s="20"/>
+      <c r="G22" s="20"/>
+      <c r="H22" s="20"/>
+      <c r="I22" s="20"/>
+      <c r="J22" s="20"/>
+      <c r="K22" s="20"/>
+      <c r="L22" s="20"/>
+      <c r="M22" s="20"/>
+      <c r="N22" s="20"/>
       <c r="O22" s="1"/>
     </row>
     <row r="23" spans="1:15" ht="23" customHeight="1">
       <c r="A23" s="1"/>
-      <c r="B23" s="20" t="s">
+      <c r="B23" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="C23" s="20"/>
+      <c r="C23" s="22"/>
       <c r="D23" s="1">
         <v>24</v>
       </c>
       <c r="E23" s="1"/>
-      <c r="F23" s="25" t="s">
+      <c r="F23" s="23" t="s">
         <v>33</v>
       </c>
-      <c r="G23" s="25"/>
-      <c r="H23" s="25"/>
-      <c r="I23" s="25"/>
-      <c r="J23" s="25"/>
-      <c r="K23" s="25"/>
-      <c r="L23" s="25"/>
-      <c r="M23" s="25"/>
-      <c r="N23" s="25"/>
+      <c r="G23" s="23"/>
+      <c r="H23" s="23"/>
+      <c r="I23" s="23"/>
+      <c r="J23" s="23"/>
+      <c r="K23" s="23"/>
+      <c r="L23" s="23"/>
+      <c r="M23" s="23"/>
+      <c r="N23" s="23"/>
       <c r="O23" s="1"/>
     </row>
     <row r="24" spans="1:15" ht="23" customHeight="1">
       <c r="A24" s="1"/>
-      <c r="B24" s="20" t="s">
+      <c r="B24" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="C24" s="20"/>
+      <c r="C24" s="22"/>
       <c r="D24" s="1">
         <v>20</v>
       </c>
       <c r="E24" s="1"/>
-      <c r="F24" s="25"/>
-      <c r="G24" s="25"/>
-      <c r="H24" s="25"/>
-      <c r="I24" s="25"/>
-      <c r="J24" s="25"/>
-      <c r="K24" s="25"/>
-      <c r="L24" s="25"/>
-      <c r="M24" s="25"/>
-      <c r="N24" s="25"/>
+      <c r="F24" s="23"/>
+      <c r="G24" s="23"/>
+      <c r="H24" s="23"/>
+      <c r="I24" s="23"/>
+      <c r="J24" s="23"/>
+      <c r="K24" s="23"/>
+      <c r="L24" s="23"/>
+      <c r="M24" s="23"/>
+      <c r="N24" s="23"/>
       <c r="O24" s="1"/>
     </row>
     <row r="25" spans="1:15" ht="23" customHeight="1">
       <c r="A25" s="1"/>
-      <c r="B25" s="20" t="s">
+      <c r="B25" s="22" t="s">
         <v>35</v>
       </c>
-      <c r="C25" s="20"/>
+      <c r="C25" s="22"/>
       <c r="D25" s="1">
         <v>40</v>
       </c>
@@ -10859,25 +10859,25 @@
     </row>
     <row r="26" spans="1:15" ht="23" customHeight="1">
       <c r="A26" s="1"/>
-      <c r="B26" s="20" t="s">
+      <c r="B26" s="22" t="s">
         <v>36</v>
       </c>
-      <c r="C26" s="20"/>
+      <c r="C26" s="22"/>
       <c r="D26" s="1">
         <v>60</v>
       </c>
       <c r="E26" s="1"/>
-      <c r="F26" s="20" t="s">
+      <c r="F26" s="22" t="s">
         <v>37</v>
       </c>
-      <c r="G26" s="20"/>
-      <c r="H26" s="20"/>
-      <c r="I26" s="20"/>
-      <c r="J26" s="20"/>
-      <c r="K26" s="20"/>
-      <c r="L26" s="20"/>
-      <c r="M26" s="20"/>
-      <c r="N26" s="20"/>
+      <c r="G26" s="22"/>
+      <c r="H26" s="22"/>
+      <c r="I26" s="22"/>
+      <c r="J26" s="22"/>
+      <c r="K26" s="22"/>
+      <c r="L26" s="22"/>
+      <c r="M26" s="22"/>
+      <c r="N26" s="22"/>
       <c r="O26" s="1"/>
     </row>
     <row r="27" spans="1:15" ht="23" customHeight="1">
@@ -10899,154 +10899,154 @@
     </row>
     <row r="28" spans="1:15" ht="23" customHeight="1">
       <c r="A28" s="1"/>
-      <c r="B28" s="23" t="s">
+      <c r="B28" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="C28" s="23"/>
-      <c r="D28" s="23"/>
-      <c r="E28" s="23"/>
-      <c r="F28" s="23"/>
-      <c r="G28" s="23"/>
-      <c r="H28" s="23"/>
-      <c r="I28" s="23"/>
-      <c r="J28" s="23"/>
-      <c r="K28" s="23"/>
-      <c r="L28" s="23"/>
-      <c r="M28" s="23"/>
-      <c r="N28" s="23"/>
+      <c r="C28" s="20"/>
+      <c r="D28" s="20"/>
+      <c r="E28" s="20"/>
+      <c r="F28" s="20"/>
+      <c r="G28" s="20"/>
+      <c r="H28" s="20"/>
+      <c r="I28" s="20"/>
+      <c r="J28" s="20"/>
+      <c r="K28" s="20"/>
+      <c r="L28" s="20"/>
+      <c r="M28" s="20"/>
+      <c r="N28" s="20"/>
       <c r="O28" s="1"/>
     </row>
     <row r="29" spans="1:15" ht="23" customHeight="1">
       <c r="A29" s="1"/>
-      <c r="B29" s="26" t="s">
+      <c r="B29" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="C29" s="26"/>
-      <c r="D29" s="26"/>
-      <c r="E29" s="26"/>
-      <c r="F29" s="26"/>
-      <c r="G29" s="26"/>
-      <c r="H29" s="26"/>
-      <c r="I29" s="26"/>
-      <c r="J29" s="26"/>
-      <c r="K29" s="26"/>
-      <c r="L29" s="26"/>
-      <c r="M29" s="26"/>
-      <c r="N29" s="26"/>
+      <c r="C29" s="19"/>
+      <c r="D29" s="19"/>
+      <c r="E29" s="19"/>
+      <c r="F29" s="19"/>
+      <c r="G29" s="19"/>
+      <c r="H29" s="19"/>
+      <c r="I29" s="19"/>
+      <c r="J29" s="19"/>
+      <c r="K29" s="19"/>
+      <c r="L29" s="19"/>
+      <c r="M29" s="19"/>
+      <c r="N29" s="19"/>
       <c r="O29" s="1"/>
     </row>
     <row r="30" spans="1:15" ht="31" customHeight="1">
       <c r="A30" s="1"/>
-      <c r="B30" s="27" t="s">
+      <c r="B30" s="21" t="s">
         <v>84</v>
       </c>
-      <c r="C30" s="27"/>
-      <c r="D30" s="27"/>
-      <c r="E30" s="27"/>
-      <c r="F30" s="27"/>
-      <c r="G30" s="27"/>
-      <c r="H30" s="27"/>
-      <c r="I30" s="27"/>
-      <c r="J30" s="27"/>
-      <c r="K30" s="27"/>
-      <c r="L30" s="27"/>
-      <c r="M30" s="27"/>
-      <c r="N30" s="27"/>
+      <c r="C30" s="21"/>
+      <c r="D30" s="21"/>
+      <c r="E30" s="21"/>
+      <c r="F30" s="21"/>
+      <c r="G30" s="21"/>
+      <c r="H30" s="21"/>
+      <c r="I30" s="21"/>
+      <c r="J30" s="21"/>
+      <c r="K30" s="21"/>
+      <c r="L30" s="21"/>
+      <c r="M30" s="21"/>
+      <c r="N30" s="21"/>
       <c r="O30" s="1"/>
     </row>
     <row r="31" spans="1:15" ht="23" customHeight="1">
       <c r="A31" s="1"/>
-      <c r="B31" s="26" t="s">
+      <c r="B31" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="C31" s="26"/>
-      <c r="D31" s="26"/>
-      <c r="E31" s="26"/>
-      <c r="F31" s="26"/>
-      <c r="G31" s="26"/>
-      <c r="H31" s="26"/>
-      <c r="I31" s="26"/>
-      <c r="J31" s="26"/>
-      <c r="K31" s="26"/>
-      <c r="L31" s="26"/>
-      <c r="M31" s="26"/>
-      <c r="N31" s="26"/>
+      <c r="C31" s="19"/>
+      <c r="D31" s="19"/>
+      <c r="E31" s="19"/>
+      <c r="F31" s="19"/>
+      <c r="G31" s="19"/>
+      <c r="H31" s="19"/>
+      <c r="I31" s="19"/>
+      <c r="J31" s="19"/>
+      <c r="K31" s="19"/>
+      <c r="L31" s="19"/>
+      <c r="M31" s="19"/>
+      <c r="N31" s="19"/>
       <c r="O31" s="1"/>
     </row>
     <row r="32" spans="1:15" ht="23" customHeight="1">
       <c r="A32" s="1"/>
-      <c r="B32" s="26" t="s">
+      <c r="B32" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="C32" s="26"/>
-      <c r="D32" s="26"/>
-      <c r="E32" s="26"/>
-      <c r="F32" s="26"/>
-      <c r="G32" s="26"/>
-      <c r="H32" s="26"/>
-      <c r="I32" s="26"/>
-      <c r="J32" s="26"/>
-      <c r="K32" s="26"/>
-      <c r="L32" s="26"/>
-      <c r="M32" s="26"/>
-      <c r="N32" s="26"/>
+      <c r="C32" s="19"/>
+      <c r="D32" s="19"/>
+      <c r="E32" s="19"/>
+      <c r="F32" s="19"/>
+      <c r="G32" s="19"/>
+      <c r="H32" s="19"/>
+      <c r="I32" s="19"/>
+      <c r="J32" s="19"/>
+      <c r="K32" s="19"/>
+      <c r="L32" s="19"/>
+      <c r="M32" s="19"/>
+      <c r="N32" s="19"/>
       <c r="O32" s="1"/>
     </row>
     <row r="33" spans="1:15" ht="23" customHeight="1">
       <c r="A33" s="1"/>
-      <c r="B33" s="26" t="s">
+      <c r="B33" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="C33" s="26"/>
-      <c r="D33" s="26"/>
-      <c r="E33" s="26"/>
-      <c r="F33" s="26"/>
-      <c r="G33" s="26"/>
-      <c r="H33" s="26"/>
-      <c r="I33" s="26"/>
-      <c r="J33" s="26"/>
-      <c r="K33" s="26"/>
-      <c r="L33" s="26"/>
-      <c r="M33" s="26"/>
-      <c r="N33" s="26"/>
+      <c r="C33" s="19"/>
+      <c r="D33" s="19"/>
+      <c r="E33" s="19"/>
+      <c r="F33" s="19"/>
+      <c r="G33" s="19"/>
+      <c r="H33" s="19"/>
+      <c r="I33" s="19"/>
+      <c r="J33" s="19"/>
+      <c r="K33" s="19"/>
+      <c r="L33" s="19"/>
+      <c r="M33" s="19"/>
+      <c r="N33" s="19"/>
       <c r="O33" s="1"/>
     </row>
     <row r="34" spans="1:15" ht="23" customHeight="1">
       <c r="A34" s="1"/>
-      <c r="B34" s="26" t="s">
+      <c r="B34" s="19" t="s">
         <v>85</v>
       </c>
-      <c r="C34" s="26"/>
-      <c r="D34" s="26"/>
-      <c r="E34" s="26"/>
-      <c r="F34" s="26"/>
-      <c r="G34" s="26"/>
-      <c r="H34" s="26"/>
-      <c r="I34" s="26"/>
-      <c r="J34" s="26"/>
-      <c r="K34" s="26"/>
-      <c r="L34" s="26"/>
-      <c r="M34" s="26"/>
-      <c r="N34" s="26"/>
+      <c r="C34" s="19"/>
+      <c r="D34" s="19"/>
+      <c r="E34" s="19"/>
+      <c r="F34" s="19"/>
+      <c r="G34" s="19"/>
+      <c r="H34" s="19"/>
+      <c r="I34" s="19"/>
+      <c r="J34" s="19"/>
+      <c r="K34" s="19"/>
+      <c r="L34" s="19"/>
+      <c r="M34" s="19"/>
+      <c r="N34" s="19"/>
       <c r="O34" s="1"/>
     </row>
     <row r="35" spans="1:15" ht="23" customHeight="1">
       <c r="A35" s="1"/>
-      <c r="B35" s="26" t="s">
+      <c r="B35" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="C35" s="26"/>
-      <c r="D35" s="26"/>
-      <c r="E35" s="26"/>
-      <c r="F35" s="26"/>
-      <c r="G35" s="26"/>
-      <c r="H35" s="26"/>
-      <c r="I35" s="26"/>
-      <c r="J35" s="26"/>
-      <c r="K35" s="26"/>
-      <c r="L35" s="26"/>
-      <c r="M35" s="26"/>
-      <c r="N35" s="26"/>
+      <c r="C35" s="19"/>
+      <c r="D35" s="19"/>
+      <c r="E35" s="19"/>
+      <c r="F35" s="19"/>
+      <c r="G35" s="19"/>
+      <c r="H35" s="19"/>
+      <c r="I35" s="19"/>
+      <c r="J35" s="19"/>
+      <c r="K35" s="19"/>
+      <c r="L35" s="19"/>
+      <c r="M35" s="19"/>
+      <c r="N35" s="19"/>
       <c r="O35" s="1"/>
     </row>
     <row r="36" spans="1:15" ht="23" customHeight="1">
@@ -11153,6 +11153,17 @@
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="B2:N2"/>
+    <mergeCell ref="B3:N3"/>
+    <mergeCell ref="D5:H5"/>
+    <mergeCell ref="J5:N5"/>
+    <mergeCell ref="B22:N22"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="F23:N24"/>
+    <mergeCell ref="F26:N26"/>
     <mergeCell ref="B33:N33"/>
     <mergeCell ref="B34:N34"/>
     <mergeCell ref="B35:N35"/>
@@ -11161,17 +11172,6 @@
     <mergeCell ref="B30:N30"/>
     <mergeCell ref="B31:N31"/>
     <mergeCell ref="B32:N32"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="F23:N24"/>
-    <mergeCell ref="F26:N26"/>
-    <mergeCell ref="B2:N2"/>
-    <mergeCell ref="B3:N3"/>
-    <mergeCell ref="D5:H5"/>
-    <mergeCell ref="J5:N5"/>
-    <mergeCell ref="B22:N22"/>
   </mergeCells>
   <phoneticPr fontId="13" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>